<commit_message>
feat(verification des INPUT): verification du PIN et du numero carte ainsi le menu
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-RayanSahbani-jnltrav.xlsx
+++ b/doc/P-P_OO-RayanSahbani-jnltrav.xlsx
@@ -5,10 +5,10 @@
   <workbookPr updateLinks="never" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML FID1\I320\Projet\OO-them-ALL\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML FID1\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67EE8600-D36F-4DA1-A4FB-9D0072C94C46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{685A6326-E499-48FA-BDC3-9E2D15E3BF29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="37">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -146,6 +146,21 @@
   </si>
   <si>
     <t>j'ai commencé à coder mon application, j'ai fais le menu</t>
+  </si>
+  <si>
+    <t>J'ai commencé par changer mon code de base car il n'était vraiment pas bien</t>
+  </si>
+  <si>
+    <t>J'ai ensuite commencer à faire le numero de carte et le pin et controler si l'utilisateur rentre bien des chiffres et non pas autre chose</t>
+  </si>
+  <si>
+    <t>Présentation</t>
+  </si>
+  <si>
+    <t>Présentation faite par le prof</t>
+  </si>
+  <si>
+    <t>J'ai commencé à essayer de voir comment je pourrai faire pour controler combien de valeur rentre l'utilisateur</t>
   </si>
 </sst>
 </file>
@@ -470,6 +485,44 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -481,44 +534,6 @@
     <xf numFmtId="14" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -853,10 +868,10 @@
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="33"/>
+      <c r="C1" s="28"/>
       <c r="D1" s="20" t="s">
         <v>1</v>
       </c>
@@ -868,10 +883,10 @@
       <c r="A2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="33"/>
+      <c r="C2" s="28"/>
       <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
@@ -883,10 +898,10 @@
       <c r="A3" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="33"/>
+      <c r="C3" s="28"/>
       <c r="D3" s="20" t="s">
         <v>6</v>
       </c>
@@ -898,12 +913,12 @@
       <c r="A4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="36"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="31"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -926,7 +941,7 @@
       <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="23">
+      <c r="B6" s="34">
         <v>46036</v>
       </c>
       <c r="C6" s="5">
@@ -941,7 +956,7 @@
       <c r="A7" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="24"/>
+      <c r="B7" s="35"/>
       <c r="C7" s="8">
         <v>3</v>
       </c>
@@ -954,7 +969,7 @@
       <c r="A8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="24"/>
+      <c r="B8" s="35"/>
       <c r="C8" s="8">
         <v>1</v>
       </c>
@@ -967,7 +982,7 @@
       <c r="A9" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="24"/>
+      <c r="B9" s="35"/>
       <c r="C9" s="8">
         <v>2</v>
       </c>
@@ -980,7 +995,7 @@
       <c r="A10" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="24"/>
+      <c r="B10" s="35"/>
       <c r="C10" s="10">
         <v>3</v>
       </c>
@@ -993,67 +1008,81 @@
       <c r="A11" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="24"/>
+      <c r="B11" s="35"/>
       <c r="C11" s="22">
         <f>SUM(C6:C10)</f>
         <v>12</v>
       </c>
-      <c r="D11" s="26"/>
-      <c r="E11" s="27"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="24"/>
     </row>
     <row r="12" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="29"/>
-      <c r="E12" s="30"/>
+      <c r="B12" s="36"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="27"/>
     </row>
     <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" s="23"/>
+        <v>30</v>
+      </c>
+      <c r="B13" s="34">
+        <v>46043</v>
+      </c>
       <c r="C13" s="5">
-        <v>1</v>
-      </c>
-      <c r="D13" s="6"/>
+        <v>2</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>32</v>
+      </c>
       <c r="E13" s="21"/>
     </row>
-    <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
-      <c r="B14" s="24"/>
+    <row r="14" spans="1:5" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="35"/>
       <c r="C14" s="8">
-        <v>1</v>
-      </c>
-      <c r="D14" s="9"/>
+        <v>5</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>33</v>
+      </c>
       <c r="E14" s="8"/>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="7"/>
-      <c r="B15" s="24"/>
+      <c r="A15" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="35"/>
       <c r="C15" s="8">
-        <v>1</v>
-      </c>
-      <c r="D15" s="9"/>
+        <v>4</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>35</v>
+      </c>
       <c r="E15" s="8"/>
     </row>
-    <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="7"/>
-      <c r="B16" s="24"/>
+    <row r="16" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="35"/>
       <c r="C16" s="8">
         <v>1</v>
       </c>
-      <c r="D16" s="9"/>
+      <c r="D16" s="9" t="s">
+        <v>36</v>
+      </c>
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="10"/>
-      <c r="B17" s="24"/>
-      <c r="C17" s="10">
-        <v>1</v>
-      </c>
+      <c r="B17" s="35"/>
+      <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
     </row>
@@ -1061,28 +1090,28 @@
       <c r="A18" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="24"/>
+      <c r="B18" s="35"/>
       <c r="C18" s="22">
         <f>SUM(C13:C17)</f>
-        <v>5</v>
-      </c>
-      <c r="D18" s="26"/>
-      <c r="E18" s="27"/>
+        <v>12</v>
+      </c>
+      <c r="D18" s="23"/>
+      <c r="E18" s="24"/>
     </row>
     <row r="19" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="30"/>
+      <c r="B19" s="36"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="27"/>
     </row>
     <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B20" s="23"/>
+      <c r="B20" s="34"/>
       <c r="C20" s="5">
         <v>1</v>
       </c>
@@ -1091,7 +1120,7 @@
     </row>
     <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7"/>
-      <c r="B21" s="24"/>
+      <c r="B21" s="35"/>
       <c r="C21" s="8">
         <v>1</v>
       </c>
@@ -1100,7 +1129,7 @@
     </row>
     <row r="22" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
-      <c r="B22" s="24"/>
+      <c r="B22" s="35"/>
       <c r="C22" s="8">
         <v>1</v>
       </c>
@@ -1109,7 +1138,7 @@
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
-      <c r="B23" s="24"/>
+      <c r="B23" s="35"/>
       <c r="C23" s="8">
         <v>1</v>
       </c>
@@ -1118,7 +1147,7 @@
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="10"/>
-      <c r="B24" s="24"/>
+      <c r="B24" s="35"/>
       <c r="C24" s="10">
         <v>1</v>
       </c>
@@ -1129,28 +1158,28 @@
       <c r="A25" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="24"/>
+      <c r="B25" s="35"/>
       <c r="C25" s="22">
         <f>SUM(C20:C24)</f>
         <v>5</v>
       </c>
-      <c r="D25" s="26"/>
-      <c r="E25" s="27"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="24"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="25"/>
-      <c r="C26" s="28"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="30"/>
+      <c r="B26" s="36"/>
+      <c r="C26" s="25"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="27"/>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B27" s="23"/>
+      <c r="B27" s="34"/>
       <c r="C27" s="5">
         <v>1</v>
       </c>
@@ -1159,7 +1188,7 @@
     </row>
     <row r="28" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
-      <c r="B28" s="24"/>
+      <c r="B28" s="35"/>
       <c r="C28" s="8">
         <v>1</v>
       </c>
@@ -1168,7 +1197,7 @@
     </row>
     <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7"/>
-      <c r="B29" s="24"/>
+      <c r="B29" s="35"/>
       <c r="C29" s="8">
         <v>1</v>
       </c>
@@ -1177,7 +1206,7 @@
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
-      <c r="B30" s="24"/>
+      <c r="B30" s="35"/>
       <c r="C30" s="8">
         <v>1</v>
       </c>
@@ -1186,7 +1215,7 @@
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="10"/>
-      <c r="B31" s="24"/>
+      <c r="B31" s="35"/>
       <c r="C31" s="10">
         <v>1</v>
       </c>
@@ -1197,28 +1226,28 @@
       <c r="A32" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B32" s="24"/>
+      <c r="B32" s="35"/>
       <c r="C32" s="22">
         <f>SUM(C27:C31)</f>
         <v>5</v>
       </c>
-      <c r="D32" s="26"/>
-      <c r="E32" s="27"/>
+      <c r="D32" s="23"/>
+      <c r="E32" s="24"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B33" s="25"/>
-      <c r="C33" s="28"/>
-      <c r="D33" s="29"/>
-      <c r="E33" s="30"/>
+      <c r="B33" s="36"/>
+      <c r="C33" s="25"/>
+      <c r="D33" s="26"/>
+      <c r="E33" s="27"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="23"/>
+      <c r="B34" s="34"/>
       <c r="C34" s="5">
         <v>1</v>
       </c>
@@ -1227,7 +1256,7 @@
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7"/>
-      <c r="B35" s="24"/>
+      <c r="B35" s="35"/>
       <c r="C35" s="8">
         <v>1</v>
       </c>
@@ -1236,7 +1265,7 @@
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7"/>
-      <c r="B36" s="24"/>
+      <c r="B36" s="35"/>
       <c r="C36" s="8">
         <v>1</v>
       </c>
@@ -1245,7 +1274,7 @@
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
-      <c r="B37" s="24"/>
+      <c r="B37" s="35"/>
       <c r="C37" s="8">
         <v>1</v>
       </c>
@@ -1254,7 +1283,7 @@
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="10"/>
-      <c r="B38" s="24"/>
+      <c r="B38" s="35"/>
       <c r="C38" s="10">
         <v>1</v>
       </c>
@@ -1265,28 +1294,28 @@
       <c r="A39" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B39" s="24"/>
+      <c r="B39" s="35"/>
       <c r="C39" s="22">
         <f>SUM(C34:C38)</f>
         <v>5</v>
       </c>
-      <c r="D39" s="26"/>
-      <c r="E39" s="27"/>
+      <c r="D39" s="23"/>
+      <c r="E39" s="24"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="25"/>
-      <c r="C40" s="28"/>
-      <c r="D40" s="29"/>
-      <c r="E40" s="30"/>
+      <c r="B40" s="36"/>
+      <c r="C40" s="25"/>
+      <c r="D40" s="26"/>
+      <c r="E40" s="27"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B41" s="23"/>
+      <c r="B41" s="34"/>
       <c r="C41" s="5">
         <v>1</v>
       </c>
@@ -1295,7 +1324,7 @@
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="7"/>
-      <c r="B42" s="24"/>
+      <c r="B42" s="35"/>
       <c r="C42" s="8">
         <v>1</v>
       </c>
@@ -1304,7 +1333,7 @@
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7"/>
-      <c r="B43" s="24"/>
+      <c r="B43" s="35"/>
       <c r="C43" s="8">
         <v>1</v>
       </c>
@@ -1313,7 +1342,7 @@
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="7"/>
-      <c r="B44" s="24"/>
+      <c r="B44" s="35"/>
       <c r="C44" s="8">
         <v>1</v>
       </c>
@@ -1322,7 +1351,7 @@
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="10"/>
-      <c r="B45" s="24"/>
+      <c r="B45" s="35"/>
       <c r="C45" s="10">
         <v>1</v>
       </c>
@@ -1333,28 +1362,28 @@
       <c r="A46" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B46" s="24"/>
+      <c r="B46" s="35"/>
       <c r="C46" s="22">
         <f>SUM(C41:C45)</f>
         <v>5</v>
       </c>
-      <c r="D46" s="26"/>
-      <c r="E46" s="27"/>
+      <c r="D46" s="23"/>
+      <c r="E46" s="24"/>
     </row>
     <row r="47" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B47" s="25"/>
-      <c r="C47" s="28"/>
-      <c r="D47" s="29"/>
-      <c r="E47" s="30"/>
+      <c r="B47" s="36"/>
+      <c r="C47" s="25"/>
+      <c r="D47" s="26"/>
+      <c r="E47" s="27"/>
     </row>
     <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="23"/>
+      <c r="B48" s="34"/>
       <c r="C48" s="5">
         <v>1</v>
       </c>
@@ -1363,7 +1392,7 @@
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
-      <c r="B49" s="24"/>
+      <c r="B49" s="35"/>
       <c r="C49" s="8">
         <v>1</v>
       </c>
@@ -1372,7 +1401,7 @@
     </row>
     <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
-      <c r="B50" s="24"/>
+      <c r="B50" s="35"/>
       <c r="C50" s="8">
         <v>1</v>
       </c>
@@ -1381,7 +1410,7 @@
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="7"/>
-      <c r="B51" s="24"/>
+      <c r="B51" s="35"/>
       <c r="C51" s="8">
         <v>1</v>
       </c>
@@ -1390,7 +1419,7 @@
     </row>
     <row r="52" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="10"/>
-      <c r="B52" s="24"/>
+      <c r="B52" s="35"/>
       <c r="C52" s="10">
         <v>1</v>
       </c>
@@ -1401,28 +1430,28 @@
       <c r="A53" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B53" s="24"/>
+      <c r="B53" s="35"/>
       <c r="C53" s="22">
         <f>SUM(C48:C52)</f>
         <v>5</v>
       </c>
-      <c r="D53" s="26"/>
-      <c r="E53" s="27"/>
+      <c r="D53" s="23"/>
+      <c r="E53" s="24"/>
     </row>
     <row r="54" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B54" s="25"/>
-      <c r="C54" s="28"/>
-      <c r="D54" s="29"/>
-      <c r="E54" s="30"/>
+      <c r="B54" s="36"/>
+      <c r="C54" s="25"/>
+      <c r="D54" s="26"/>
+      <c r="E54" s="27"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B55" s="23"/>
+      <c r="B55" s="34"/>
       <c r="C55" s="5">
         <v>1</v>
       </c>
@@ -1431,7 +1460,7 @@
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="7"/>
-      <c r="B56" s="24"/>
+      <c r="B56" s="35"/>
       <c r="C56" s="8">
         <v>1</v>
       </c>
@@ -1440,7 +1469,7 @@
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="7"/>
-      <c r="B57" s="24"/>
+      <c r="B57" s="35"/>
       <c r="C57" s="8">
         <v>1</v>
       </c>
@@ -1449,7 +1478,7 @@
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="24"/>
+      <c r="B58" s="35"/>
       <c r="C58" s="8">
         <v>1</v>
       </c>
@@ -1458,7 +1487,7 @@
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="10"/>
-      <c r="B59" s="24"/>
+      <c r="B59" s="35"/>
       <c r="C59" s="10">
         <v>1</v>
       </c>
@@ -1469,28 +1498,28 @@
       <c r="A60" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B60" s="24"/>
+      <c r="B60" s="35"/>
       <c r="C60" s="22">
         <f>SUM(C55:C59)</f>
         <v>5</v>
       </c>
-      <c r="D60" s="26"/>
-      <c r="E60" s="27"/>
+      <c r="D60" s="23"/>
+      <c r="E60" s="24"/>
     </row>
     <row r="61" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B61" s="25"/>
-      <c r="C61" s="28"/>
-      <c r="D61" s="29"/>
-      <c r="E61" s="30"/>
+      <c r="B61" s="36"/>
+      <c r="C61" s="25"/>
+      <c r="D61" s="26"/>
+      <c r="E61" s="27"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B62" s="23"/>
+      <c r="B62" s="34"/>
       <c r="C62" s="5">
         <v>1</v>
       </c>
@@ -1499,7 +1528,7 @@
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
-      <c r="B63" s="24"/>
+      <c r="B63" s="35"/>
       <c r="C63" s="8">
         <v>1</v>
       </c>
@@ -1508,7 +1537,7 @@
     </row>
     <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="24"/>
+      <c r="B64" s="35"/>
       <c r="C64" s="8">
         <v>1</v>
       </c>
@@ -1517,7 +1546,7 @@
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="7"/>
-      <c r="B65" s="24"/>
+      <c r="B65" s="35"/>
       <c r="C65" s="8">
         <v>1</v>
       </c>
@@ -1526,7 +1555,7 @@
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="24"/>
+      <c r="B66" s="35"/>
       <c r="C66" s="10">
         <v>1</v>
       </c>
@@ -1537,28 +1566,28 @@
       <c r="A67" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B67" s="24"/>
+      <c r="B67" s="35"/>
       <c r="C67" s="22">
         <f>SUM(C62:C66)</f>
         <v>5</v>
       </c>
-      <c r="D67" s="26"/>
-      <c r="E67" s="27"/>
+      <c r="D67" s="23"/>
+      <c r="E67" s="24"/>
     </row>
     <row r="68" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B68" s="25"/>
-      <c r="C68" s="28"/>
-      <c r="D68" s="29"/>
-      <c r="E68" s="30"/>
+      <c r="B68" s="36"/>
+      <c r="C68" s="25"/>
+      <c r="D68" s="26"/>
+      <c r="E68" s="27"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B69" s="23"/>
+      <c r="B69" s="34"/>
       <c r="C69" s="5">
         <v>1</v>
       </c>
@@ -1567,7 +1596,7 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="7"/>
-      <c r="B70" s="24"/>
+      <c r="B70" s="35"/>
       <c r="C70" s="8">
         <v>1</v>
       </c>
@@ -1576,7 +1605,7 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="7"/>
-      <c r="B71" s="24"/>
+      <c r="B71" s="35"/>
       <c r="C71" s="8">
         <v>1</v>
       </c>
@@ -1585,7 +1614,7 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="7"/>
-      <c r="B72" s="24"/>
+      <c r="B72" s="35"/>
       <c r="C72" s="8">
         <v>1</v>
       </c>
@@ -1594,7 +1623,7 @@
     </row>
     <row r="73" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="10"/>
-      <c r="B73" s="24"/>
+      <c r="B73" s="35"/>
       <c r="C73" s="10">
         <v>1</v>
       </c>
@@ -1605,28 +1634,28 @@
       <c r="A74" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B74" s="24"/>
+      <c r="B74" s="35"/>
       <c r="C74" s="22">
         <f>SUM(C69:C73)</f>
         <v>5</v>
       </c>
-      <c r="D74" s="26"/>
-      <c r="E74" s="27"/>
+      <c r="D74" s="23"/>
+      <c r="E74" s="24"/>
     </row>
     <row r="75" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B75" s="25"/>
-      <c r="C75" s="28"/>
-      <c r="D75" s="29"/>
-      <c r="E75" s="30"/>
+      <c r="B75" s="36"/>
+      <c r="C75" s="25"/>
+      <c r="D75" s="26"/>
+      <c r="E75" s="27"/>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B76" s="23"/>
+      <c r="B76" s="34"/>
       <c r="C76" s="5">
         <v>1</v>
       </c>
@@ -1635,7 +1664,7 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="7"/>
-      <c r="B77" s="24"/>
+      <c r="B77" s="35"/>
       <c r="C77" s="8">
         <v>1</v>
       </c>
@@ -1644,7 +1673,7 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="7"/>
-      <c r="B78" s="24"/>
+      <c r="B78" s="35"/>
       <c r="C78" s="8">
         <v>1</v>
       </c>
@@ -1653,7 +1682,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="7"/>
-      <c r="B79" s="24"/>
+      <c r="B79" s="35"/>
       <c r="C79" s="8">
         <v>1</v>
       </c>
@@ -1662,7 +1691,7 @@
     </row>
     <row r="80" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="10"/>
-      <c r="B80" s="24"/>
+      <c r="B80" s="35"/>
       <c r="C80" s="10">
         <v>1</v>
       </c>
@@ -1673,28 +1702,28 @@
       <c r="A81" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B81" s="24"/>
+      <c r="B81" s="35"/>
       <c r="C81" s="22">
         <f>SUM(C76:C80)</f>
         <v>5</v>
       </c>
-      <c r="D81" s="26"/>
-      <c r="E81" s="27"/>
+      <c r="D81" s="23"/>
+      <c r="E81" s="24"/>
     </row>
     <row r="82" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B82" s="25"/>
-      <c r="C82" s="28"/>
-      <c r="D82" s="29"/>
-      <c r="E82" s="30"/>
+      <c r="B82" s="36"/>
+      <c r="C82" s="25"/>
+      <c r="D82" s="26"/>
+      <c r="E82" s="27"/>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B83" s="23"/>
+      <c r="B83" s="34"/>
       <c r="C83" s="5">
         <v>1</v>
       </c>
@@ -1703,7 +1732,7 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="7"/>
-      <c r="B84" s="24"/>
+      <c r="B84" s="35"/>
       <c r="C84" s="8">
         <v>1</v>
       </c>
@@ -1712,7 +1741,7 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="7"/>
-      <c r="B85" s="24"/>
+      <c r="B85" s="35"/>
       <c r="C85" s="8">
         <v>1</v>
       </c>
@@ -1721,7 +1750,7 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="7"/>
-      <c r="B86" s="24"/>
+      <c r="B86" s="35"/>
       <c r="C86" s="8">
         <v>1</v>
       </c>
@@ -1730,7 +1759,7 @@
     </row>
     <row r="87" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="10"/>
-      <c r="B87" s="24"/>
+      <c r="B87" s="35"/>
       <c r="C87" s="10">
         <v>1</v>
       </c>
@@ -1741,31 +1770,31 @@
       <c r="A88" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B88" s="24"/>
+      <c r="B88" s="35"/>
       <c r="C88" s="22">
         <f>SUM(C83:C87)</f>
         <v>5</v>
       </c>
-      <c r="D88" s="26"/>
-      <c r="E88" s="27"/>
+      <c r="D88" s="23"/>
+      <c r="E88" s="24"/>
     </row>
     <row r="89" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B89" s="25"/>
-      <c r="C89" s="28"/>
-      <c r="D89" s="29"/>
-      <c r="E89" s="30"/>
+      <c r="B89" s="36"/>
+      <c r="C89" s="25"/>
+      <c r="D89" s="26"/>
+      <c r="E89" s="27"/>
     </row>
     <row r="90" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="31" t="s">
+      <c r="A90" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="B90" s="32"/>
+      <c r="B90" s="33"/>
       <c r="C90" s="13">
         <f>MROUND(SUM(C6:C89) /8,0.2)</f>
-        <v>16.8</v>
+        <v>18.600000000000001</v>
       </c>
       <c r="D90" s="14"/>
       <c r="E90" s="15"/>
@@ -1780,17 +1809,37 @@
     </row>
   </sheetData>
   <mergeCells count="41">
+    <mergeCell ref="D81:E81"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="B83:B89"/>
+    <mergeCell ref="D88:E88"/>
+    <mergeCell ref="C89:E89"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="B69:B75"/>
+    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="C75:E75"/>
+    <mergeCell ref="B27:B33"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="C47:E47"/>
+    <mergeCell ref="A90:B90"/>
+    <mergeCell ref="B34:B40"/>
+    <mergeCell ref="B41:B47"/>
+    <mergeCell ref="B48:B54"/>
+    <mergeCell ref="B55:B61"/>
+    <mergeCell ref="B62:B68"/>
+    <mergeCell ref="B76:B82"/>
     <mergeCell ref="D60:E60"/>
     <mergeCell ref="C61:E61"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="A90:B90"/>
-    <mergeCell ref="B34:B40"/>
-    <mergeCell ref="B41:B47"/>
-    <mergeCell ref="B48:B54"/>
-    <mergeCell ref="B55:B61"/>
     <mergeCell ref="C54:E54"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="C12:E12"/>
@@ -1801,26 +1850,6 @@
     <mergeCell ref="B20:B26"/>
     <mergeCell ref="D25:E25"/>
     <mergeCell ref="C26:E26"/>
-    <mergeCell ref="B27:B33"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="B62:B68"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="B69:B75"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="C75:E75"/>
-    <mergeCell ref="B76:B82"/>
-    <mergeCell ref="D81:E81"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="B83:B89"/>
-    <mergeCell ref="D88:E88"/>
-    <mergeCell ref="C89:E89"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C11 B13 C13:C18 B20 C20:C25 B27 C27:C32 B34 C34:C39 B41 C41:C46 B48 C48:C53 B55 C55:C60 B62 C62:C67 B69 C69:C74 B76 C76:C81 B83 C83:C88" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -1839,18 +1868,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2016,18 +2045,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
(v1 procédural):le CDC est respecté et la v1 est prête pour le release
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-RayanSahbani-jnltrav.xlsx
+++ b/doc/P-P_OO-RayanSahbani-jnltrav.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML FID1\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{685A6326-E499-48FA-BDC3-9E2D15E3BF29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF6E9B29-7BD5-4585-B9D2-6C58C21EA1F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="42">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -161,6 +161,21 @@
   </si>
   <si>
     <t>J'ai commencé à essayer de voir comment je pourrai faire pour controler combien de valeur rentre l'utilisateur</t>
+  </si>
+  <si>
+    <t>Visual Studio</t>
+  </si>
+  <si>
+    <t>j'ai fais le deuxième menu de mon bancomate, la fonction pour verifier les codes, et retirer</t>
+  </si>
+  <si>
+    <t>J'ai fais la fonction consulter solde qui permet de consulter le sole et la fonction recu qui ma pris un peu de temps.</t>
+  </si>
+  <si>
+    <t>Je suis revenue sur ma fonction retirer car elle avait plusieurs failles comme par exemple l'utilisateur pouvait retirer plus que ce qu'il avait, et je suis aussi revenu sur le menu pour faire un tableau</t>
+  </si>
+  <si>
+    <t>je suis aussi revenu sur le menu pour faire un tableau</t>
   </si>
 </sst>
 </file>
@@ -505,24 +520,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -534,6 +531,24 @@
     <xf numFmtId="14" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -868,10 +883,10 @@
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="28"/>
+      <c r="C1" s="33"/>
       <c r="D1" s="20" t="s">
         <v>1</v>
       </c>
@@ -883,10 +898,10 @@
       <c r="A2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="28"/>
+      <c r="C2" s="33"/>
       <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
@@ -898,10 +913,10 @@
       <c r="A3" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="28"/>
+      <c r="C3" s="33"/>
       <c r="D3" s="20" t="s">
         <v>6</v>
       </c>
@@ -913,12 +928,12 @@
       <c r="A4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="31"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="36"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -941,7 +956,7 @@
       <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="34">
+      <c r="B6" s="28">
         <v>46036</v>
       </c>
       <c r="C6" s="5">
@@ -956,7 +971,7 @@
       <c r="A7" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="35"/>
+      <c r="B7" s="29"/>
       <c r="C7" s="8">
         <v>3</v>
       </c>
@@ -969,7 +984,7 @@
       <c r="A8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="35"/>
+      <c r="B8" s="29"/>
       <c r="C8" s="8">
         <v>1</v>
       </c>
@@ -982,7 +997,7 @@
       <c r="A9" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="35"/>
+      <c r="B9" s="29"/>
       <c r="C9" s="8">
         <v>2</v>
       </c>
@@ -995,7 +1010,7 @@
       <c r="A10" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="35"/>
+      <c r="B10" s="29"/>
       <c r="C10" s="10">
         <v>3</v>
       </c>
@@ -1008,7 +1023,7 @@
       <c r="A11" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="35"/>
+      <c r="B11" s="29"/>
       <c r="C11" s="22">
         <f>SUM(C6:C10)</f>
         <v>12</v>
@@ -1020,7 +1035,7 @@
       <c r="A12" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="36"/>
+      <c r="B12" s="30"/>
       <c r="C12" s="25"/>
       <c r="D12" s="26"/>
       <c r="E12" s="27"/>
@@ -1029,7 +1044,7 @@
       <c r="A13" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="34">
+      <c r="B13" s="28">
         <v>46043</v>
       </c>
       <c r="C13" s="5">
@@ -1044,7 +1059,7 @@
       <c r="A14" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="35"/>
+      <c r="B14" s="29"/>
       <c r="C14" s="8">
         <v>5</v>
       </c>
@@ -1057,7 +1072,7 @@
       <c r="A15" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="35"/>
+      <c r="B15" s="29"/>
       <c r="C15" s="8">
         <v>4</v>
       </c>
@@ -1070,7 +1085,7 @@
       <c r="A16" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="35"/>
+      <c r="B16" s="29"/>
       <c r="C16" s="8">
         <v>1</v>
       </c>
@@ -1081,7 +1096,7 @@
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="10"/>
-      <c r="B17" s="35"/>
+      <c r="B17" s="29"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1090,7 +1105,7 @@
       <c r="A18" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="35"/>
+      <c r="B18" s="29"/>
       <c r="C18" s="22">
         <f>SUM(C13:C17)</f>
         <v>12</v>
@@ -1102,55 +1117,65 @@
       <c r="A19" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="36"/>
+      <c r="B19" s="30"/>
       <c r="C19" s="25"/>
       <c r="D19" s="26"/>
       <c r="E19" s="27"/>
     </row>
-    <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B20" s="34"/>
+        <v>37</v>
+      </c>
+      <c r="B20" s="28">
+        <v>46050</v>
+      </c>
       <c r="C20" s="5">
-        <v>1</v>
-      </c>
-      <c r="D20" s="6"/>
+        <v>5</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>38</v>
+      </c>
       <c r="E20" s="21"/>
     </row>
-    <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="7"/>
-      <c r="B21" s="35"/>
+    <row r="21" spans="1:5" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" s="29"/>
       <c r="C21" s="8">
-        <v>1</v>
-      </c>
-      <c r="D21" s="9"/>
+        <v>3</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>39</v>
+      </c>
       <c r="E21" s="8"/>
     </row>
-    <row r="22" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
-      <c r="B22" s="35"/>
+      <c r="B22" s="29"/>
       <c r="C22" s="8">
-        <v>1</v>
-      </c>
-      <c r="D22" s="9"/>
+        <v>2</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>40</v>
+      </c>
       <c r="E22" s="8"/>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
-      <c r="B23" s="35"/>
+      <c r="B23" s="29"/>
       <c r="C23" s="8">
-        <v>1</v>
-      </c>
-      <c r="D23" s="9"/>
+        <v>2</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>41</v>
+      </c>
       <c r="E23" s="8"/>
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="10"/>
-      <c r="B24" s="35"/>
-      <c r="C24" s="10">
-        <v>1</v>
-      </c>
+      <c r="B24" s="29"/>
+      <c r="C24" s="10"/>
       <c r="D24" s="11"/>
       <c r="E24" s="10"/>
     </row>
@@ -1158,10 +1183,10 @@
       <c r="A25" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="35"/>
+      <c r="B25" s="29"/>
       <c r="C25" s="22">
         <f>SUM(C20:C24)</f>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D25" s="23"/>
       <c r="E25" s="24"/>
@@ -1170,7 +1195,7 @@
       <c r="A26" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="36"/>
+      <c r="B26" s="30"/>
       <c r="C26" s="25"/>
       <c r="D26" s="26"/>
       <c r="E26" s="27"/>
@@ -1179,7 +1204,7 @@
       <c r="A27" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B27" s="34"/>
+      <c r="B27" s="28"/>
       <c r="C27" s="5">
         <v>1</v>
       </c>
@@ -1188,7 +1213,7 @@
     </row>
     <row r="28" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
-      <c r="B28" s="35"/>
+      <c r="B28" s="29"/>
       <c r="C28" s="8">
         <v>1</v>
       </c>
@@ -1197,7 +1222,7 @@
     </row>
     <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7"/>
-      <c r="B29" s="35"/>
+      <c r="B29" s="29"/>
       <c r="C29" s="8">
         <v>1</v>
       </c>
@@ -1206,7 +1231,7 @@
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
-      <c r="B30" s="35"/>
+      <c r="B30" s="29"/>
       <c r="C30" s="8">
         <v>1</v>
       </c>
@@ -1215,7 +1240,7 @@
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="10"/>
-      <c r="B31" s="35"/>
+      <c r="B31" s="29"/>
       <c r="C31" s="10">
         <v>1</v>
       </c>
@@ -1226,7 +1251,7 @@
       <c r="A32" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B32" s="35"/>
+      <c r="B32" s="29"/>
       <c r="C32" s="22">
         <f>SUM(C27:C31)</f>
         <v>5</v>
@@ -1238,7 +1263,7 @@
       <c r="A33" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B33" s="36"/>
+      <c r="B33" s="30"/>
       <c r="C33" s="25"/>
       <c r="D33" s="26"/>
       <c r="E33" s="27"/>
@@ -1247,7 +1272,7 @@
       <c r="A34" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="34"/>
+      <c r="B34" s="28"/>
       <c r="C34" s="5">
         <v>1</v>
       </c>
@@ -1256,7 +1281,7 @@
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7"/>
-      <c r="B35" s="35"/>
+      <c r="B35" s="29"/>
       <c r="C35" s="8">
         <v>1</v>
       </c>
@@ -1265,7 +1290,7 @@
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7"/>
-      <c r="B36" s="35"/>
+      <c r="B36" s="29"/>
       <c r="C36" s="8">
         <v>1</v>
       </c>
@@ -1274,7 +1299,7 @@
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
-      <c r="B37" s="35"/>
+      <c r="B37" s="29"/>
       <c r="C37" s="8">
         <v>1</v>
       </c>
@@ -1283,7 +1308,7 @@
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="10"/>
-      <c r="B38" s="35"/>
+      <c r="B38" s="29"/>
       <c r="C38" s="10">
         <v>1</v>
       </c>
@@ -1294,7 +1319,7 @@
       <c r="A39" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B39" s="35"/>
+      <c r="B39" s="29"/>
       <c r="C39" s="22">
         <f>SUM(C34:C38)</f>
         <v>5</v>
@@ -1306,7 +1331,7 @@
       <c r="A40" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="36"/>
+      <c r="B40" s="30"/>
       <c r="C40" s="25"/>
       <c r="D40" s="26"/>
       <c r="E40" s="27"/>
@@ -1315,7 +1340,7 @@
       <c r="A41" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B41" s="34"/>
+      <c r="B41" s="28"/>
       <c r="C41" s="5">
         <v>1</v>
       </c>
@@ -1324,7 +1349,7 @@
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="7"/>
-      <c r="B42" s="35"/>
+      <c r="B42" s="29"/>
       <c r="C42" s="8">
         <v>1</v>
       </c>
@@ -1333,7 +1358,7 @@
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7"/>
-      <c r="B43" s="35"/>
+      <c r="B43" s="29"/>
       <c r="C43" s="8">
         <v>1</v>
       </c>
@@ -1342,7 +1367,7 @@
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="7"/>
-      <c r="B44" s="35"/>
+      <c r="B44" s="29"/>
       <c r="C44" s="8">
         <v>1</v>
       </c>
@@ -1351,7 +1376,7 @@
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="10"/>
-      <c r="B45" s="35"/>
+      <c r="B45" s="29"/>
       <c r="C45" s="10">
         <v>1</v>
       </c>
@@ -1362,7 +1387,7 @@
       <c r="A46" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B46" s="35"/>
+      <c r="B46" s="29"/>
       <c r="C46" s="22">
         <f>SUM(C41:C45)</f>
         <v>5</v>
@@ -1374,7 +1399,7 @@
       <c r="A47" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B47" s="36"/>
+      <c r="B47" s="30"/>
       <c r="C47" s="25"/>
       <c r="D47" s="26"/>
       <c r="E47" s="27"/>
@@ -1383,7 +1408,7 @@
       <c r="A48" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="34"/>
+      <c r="B48" s="28"/>
       <c r="C48" s="5">
         <v>1</v>
       </c>
@@ -1392,7 +1417,7 @@
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
-      <c r="B49" s="35"/>
+      <c r="B49" s="29"/>
       <c r="C49" s="8">
         <v>1</v>
       </c>
@@ -1401,7 +1426,7 @@
     </row>
     <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
-      <c r="B50" s="35"/>
+      <c r="B50" s="29"/>
       <c r="C50" s="8">
         <v>1</v>
       </c>
@@ -1410,7 +1435,7 @@
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="7"/>
-      <c r="B51" s="35"/>
+      <c r="B51" s="29"/>
       <c r="C51" s="8">
         <v>1</v>
       </c>
@@ -1419,7 +1444,7 @@
     </row>
     <row r="52" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="10"/>
-      <c r="B52" s="35"/>
+      <c r="B52" s="29"/>
       <c r="C52" s="10">
         <v>1</v>
       </c>
@@ -1430,7 +1455,7 @@
       <c r="A53" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B53" s="35"/>
+      <c r="B53" s="29"/>
       <c r="C53" s="22">
         <f>SUM(C48:C52)</f>
         <v>5</v>
@@ -1442,7 +1467,7 @@
       <c r="A54" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B54" s="36"/>
+      <c r="B54" s="30"/>
       <c r="C54" s="25"/>
       <c r="D54" s="26"/>
       <c r="E54" s="27"/>
@@ -1451,7 +1476,7 @@
       <c r="A55" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B55" s="34"/>
+      <c r="B55" s="28"/>
       <c r="C55" s="5">
         <v>1</v>
       </c>
@@ -1460,7 +1485,7 @@
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="7"/>
-      <c r="B56" s="35"/>
+      <c r="B56" s="29"/>
       <c r="C56" s="8">
         <v>1</v>
       </c>
@@ -1469,7 +1494,7 @@
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="7"/>
-      <c r="B57" s="35"/>
+      <c r="B57" s="29"/>
       <c r="C57" s="8">
         <v>1</v>
       </c>
@@ -1478,7 +1503,7 @@
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="35"/>
+      <c r="B58" s="29"/>
       <c r="C58" s="8">
         <v>1</v>
       </c>
@@ -1487,7 +1512,7 @@
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="10"/>
-      <c r="B59" s="35"/>
+      <c r="B59" s="29"/>
       <c r="C59" s="10">
         <v>1</v>
       </c>
@@ -1498,7 +1523,7 @@
       <c r="A60" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B60" s="35"/>
+      <c r="B60" s="29"/>
       <c r="C60" s="22">
         <f>SUM(C55:C59)</f>
         <v>5</v>
@@ -1510,7 +1535,7 @@
       <c r="A61" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B61" s="36"/>
+      <c r="B61" s="30"/>
       <c r="C61" s="25"/>
       <c r="D61" s="26"/>
       <c r="E61" s="27"/>
@@ -1519,7 +1544,7 @@
       <c r="A62" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B62" s="34"/>
+      <c r="B62" s="28"/>
       <c r="C62" s="5">
         <v>1</v>
       </c>
@@ -1528,7 +1553,7 @@
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
-      <c r="B63" s="35"/>
+      <c r="B63" s="29"/>
       <c r="C63" s="8">
         <v>1</v>
       </c>
@@ -1537,7 +1562,7 @@
     </row>
     <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="35"/>
+      <c r="B64" s="29"/>
       <c r="C64" s="8">
         <v>1</v>
       </c>
@@ -1546,7 +1571,7 @@
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="7"/>
-      <c r="B65" s="35"/>
+      <c r="B65" s="29"/>
       <c r="C65" s="8">
         <v>1</v>
       </c>
@@ -1555,7 +1580,7 @@
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="35"/>
+      <c r="B66" s="29"/>
       <c r="C66" s="10">
         <v>1</v>
       </c>
@@ -1566,7 +1591,7 @@
       <c r="A67" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B67" s="35"/>
+      <c r="B67" s="29"/>
       <c r="C67" s="22">
         <f>SUM(C62:C66)</f>
         <v>5</v>
@@ -1578,7 +1603,7 @@
       <c r="A68" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B68" s="36"/>
+      <c r="B68" s="30"/>
       <c r="C68" s="25"/>
       <c r="D68" s="26"/>
       <c r="E68" s="27"/>
@@ -1587,7 +1612,7 @@
       <c r="A69" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B69" s="34"/>
+      <c r="B69" s="28"/>
       <c r="C69" s="5">
         <v>1</v>
       </c>
@@ -1596,7 +1621,7 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="7"/>
-      <c r="B70" s="35"/>
+      <c r="B70" s="29"/>
       <c r="C70" s="8">
         <v>1</v>
       </c>
@@ -1605,7 +1630,7 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="7"/>
-      <c r="B71" s="35"/>
+      <c r="B71" s="29"/>
       <c r="C71" s="8">
         <v>1</v>
       </c>
@@ -1614,7 +1639,7 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="7"/>
-      <c r="B72" s="35"/>
+      <c r="B72" s="29"/>
       <c r="C72" s="8">
         <v>1</v>
       </c>
@@ -1623,7 +1648,7 @@
     </row>
     <row r="73" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="10"/>
-      <c r="B73" s="35"/>
+      <c r="B73" s="29"/>
       <c r="C73" s="10">
         <v>1</v>
       </c>
@@ -1634,7 +1659,7 @@
       <c r="A74" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B74" s="35"/>
+      <c r="B74" s="29"/>
       <c r="C74" s="22">
         <f>SUM(C69:C73)</f>
         <v>5</v>
@@ -1646,7 +1671,7 @@
       <c r="A75" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B75" s="36"/>
+      <c r="B75" s="30"/>
       <c r="C75" s="25"/>
       <c r="D75" s="26"/>
       <c r="E75" s="27"/>
@@ -1655,7 +1680,7 @@
       <c r="A76" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B76" s="34"/>
+      <c r="B76" s="28"/>
       <c r="C76" s="5">
         <v>1</v>
       </c>
@@ -1664,7 +1689,7 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="7"/>
-      <c r="B77" s="35"/>
+      <c r="B77" s="29"/>
       <c r="C77" s="8">
         <v>1</v>
       </c>
@@ -1673,7 +1698,7 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="7"/>
-      <c r="B78" s="35"/>
+      <c r="B78" s="29"/>
       <c r="C78" s="8">
         <v>1</v>
       </c>
@@ -1682,7 +1707,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="7"/>
-      <c r="B79" s="35"/>
+      <c r="B79" s="29"/>
       <c r="C79" s="8">
         <v>1</v>
       </c>
@@ -1691,7 +1716,7 @@
     </row>
     <row r="80" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="10"/>
-      <c r="B80" s="35"/>
+      <c r="B80" s="29"/>
       <c r="C80" s="10">
         <v>1</v>
       </c>
@@ -1702,7 +1727,7 @@
       <c r="A81" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B81" s="35"/>
+      <c r="B81" s="29"/>
       <c r="C81" s="22">
         <f>SUM(C76:C80)</f>
         <v>5</v>
@@ -1714,7 +1739,7 @@
       <c r="A82" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B82" s="36"/>
+      <c r="B82" s="30"/>
       <c r="C82" s="25"/>
       <c r="D82" s="26"/>
       <c r="E82" s="27"/>
@@ -1723,7 +1748,7 @@
       <c r="A83" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B83" s="34"/>
+      <c r="B83" s="28"/>
       <c r="C83" s="5">
         <v>1</v>
       </c>
@@ -1732,7 +1757,7 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="7"/>
-      <c r="B84" s="35"/>
+      <c r="B84" s="29"/>
       <c r="C84" s="8">
         <v>1</v>
       </c>
@@ -1741,7 +1766,7 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="7"/>
-      <c r="B85" s="35"/>
+      <c r="B85" s="29"/>
       <c r="C85" s="8">
         <v>1</v>
       </c>
@@ -1750,7 +1775,7 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="7"/>
-      <c r="B86" s="35"/>
+      <c r="B86" s="29"/>
       <c r="C86" s="8">
         <v>1</v>
       </c>
@@ -1759,7 +1784,7 @@
     </row>
     <row r="87" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="10"/>
-      <c r="B87" s="35"/>
+      <c r="B87" s="29"/>
       <c r="C87" s="10">
         <v>1</v>
       </c>
@@ -1770,7 +1795,7 @@
       <c r="A88" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B88" s="35"/>
+      <c r="B88" s="29"/>
       <c r="C88" s="22">
         <f>SUM(C83:C87)</f>
         <v>5</v>
@@ -1782,19 +1807,19 @@
       <c r="A89" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B89" s="36"/>
+      <c r="B89" s="30"/>
       <c r="C89" s="25"/>
       <c r="D89" s="26"/>
       <c r="E89" s="27"/>
     </row>
     <row r="90" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="32" t="s">
+      <c r="A90" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="B90" s="33"/>
+      <c r="B90" s="32"/>
       <c r="C90" s="13">
         <f>MROUND(SUM(C6:C89) /8,0.2)</f>
-        <v>18.600000000000001</v>
+        <v>20.200000000000003</v>
       </c>
       <c r="D90" s="14"/>
       <c r="E90" s="15"/>
@@ -1809,31 +1834,6 @@
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="D81:E81"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="B83:B89"/>
-    <mergeCell ref="D88:E88"/>
-    <mergeCell ref="C89:E89"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="B69:B75"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="C75:E75"/>
-    <mergeCell ref="B27:B33"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="A90:B90"/>
-    <mergeCell ref="B34:B40"/>
-    <mergeCell ref="B41:B47"/>
-    <mergeCell ref="B48:B54"/>
-    <mergeCell ref="B55:B61"/>
-    <mergeCell ref="B62:B68"/>
-    <mergeCell ref="B76:B82"/>
     <mergeCell ref="D60:E60"/>
     <mergeCell ref="C61:E61"/>
     <mergeCell ref="B1:C1"/>
@@ -1850,6 +1850,31 @@
     <mergeCell ref="B20:B26"/>
     <mergeCell ref="D25:E25"/>
     <mergeCell ref="C26:E26"/>
+    <mergeCell ref="A90:B90"/>
+    <mergeCell ref="B34:B40"/>
+    <mergeCell ref="B41:B47"/>
+    <mergeCell ref="B48:B54"/>
+    <mergeCell ref="B55:B61"/>
+    <mergeCell ref="B62:B68"/>
+    <mergeCell ref="B76:B82"/>
+    <mergeCell ref="B27:B33"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="C47:E47"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="B69:B75"/>
+    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="C75:E75"/>
+    <mergeCell ref="D81:E81"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="B83:B89"/>
+    <mergeCell ref="D88:E88"/>
+    <mergeCell ref="C89:E89"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C11 B13 C13:C18 B20 C20:C25 B27 C27:C32 B34 C34:C39 B41 C41:C46 B48 C48:C53 B55 C55:C60 B62 C62:C67 B69 C69:C74 B76 C76:C81 B83 C83:C88" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -1868,18 +1893,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2045,18 +2070,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
chore(Visuel et commentaire): amelioration du visiuel, verification du retrait et ajout de commentaire
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-RayanSahbani-jnltrav.xlsx
+++ b/doc/P-P_OO-RayanSahbani-jnltrav.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML FID1\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF368B8F-5D31-4C0D-8630-54EB00C26A35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{074084A4-7BFF-4A42-81C0-E7641A54EE03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="49">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -188,6 +188,15 @@
   </si>
   <si>
     <t xml:space="preserve">J'ai fais la classe TransactionProcessor et AuthentificationManager qui m'ont pris du temps car j'ai eu plusieurs problème </t>
+  </si>
+  <si>
+    <t>J'ai commenté mon code et j'ai fais l'entete.</t>
+  </si>
+  <si>
+    <t>J'ai amelioré ma classe withDraw pour verifier ce que entre l'utilisateur</t>
+  </si>
+  <si>
+    <t>J'ai amélioré le visuel de mon code et j'ai aussi fais des tests pour voir si tout fonctionne bien.</t>
   </si>
 </sst>
 </file>
@@ -532,18 +541,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -561,6 +558,18 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -895,10 +904,10 @@
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="28"/>
+      <c r="C1" s="33"/>
       <c r="D1" s="20" t="s">
         <v>1</v>
       </c>
@@ -910,10 +919,10 @@
       <c r="A2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="28"/>
+      <c r="C2" s="33"/>
       <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
@@ -925,10 +934,10 @@
       <c r="A3" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="28"/>
+      <c r="C3" s="33"/>
       <c r="D3" s="20" t="s">
         <v>6</v>
       </c>
@@ -940,12 +949,12 @@
       <c r="A4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="31"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="36"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -968,7 +977,7 @@
       <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="32">
+      <c r="B6" s="28">
         <v>46036</v>
       </c>
       <c r="C6" s="5">
@@ -983,7 +992,7 @@
       <c r="A7" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="33"/>
+      <c r="B7" s="29"/>
       <c r="C7" s="8">
         <v>3</v>
       </c>
@@ -996,7 +1005,7 @@
       <c r="A8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="33"/>
+      <c r="B8" s="29"/>
       <c r="C8" s="8">
         <v>1</v>
       </c>
@@ -1009,7 +1018,7 @@
       <c r="A9" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="33"/>
+      <c r="B9" s="29"/>
       <c r="C9" s="8">
         <v>2</v>
       </c>
@@ -1022,7 +1031,7 @@
       <c r="A10" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="33"/>
+      <c r="B10" s="29"/>
       <c r="C10" s="10">
         <v>3</v>
       </c>
@@ -1035,7 +1044,7 @@
       <c r="A11" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="33"/>
+      <c r="B11" s="29"/>
       <c r="C11" s="22">
         <f>SUM(C6:C10)</f>
         <v>12</v>
@@ -1047,7 +1056,7 @@
       <c r="A12" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="34"/>
+      <c r="B12" s="30"/>
       <c r="C12" s="25"/>
       <c r="D12" s="26"/>
       <c r="E12" s="27"/>
@@ -1056,7 +1065,7 @@
       <c r="A13" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="32">
+      <c r="B13" s="28">
         <v>46043</v>
       </c>
       <c r="C13" s="5">
@@ -1071,7 +1080,7 @@
       <c r="A14" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="33"/>
+      <c r="B14" s="29"/>
       <c r="C14" s="8">
         <v>5</v>
       </c>
@@ -1084,7 +1093,7 @@
       <c r="A15" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="33"/>
+      <c r="B15" s="29"/>
       <c r="C15" s="8">
         <v>4</v>
       </c>
@@ -1097,7 +1106,7 @@
       <c r="A16" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="33"/>
+      <c r="B16" s="29"/>
       <c r="C16" s="8">
         <v>1</v>
       </c>
@@ -1108,7 +1117,7 @@
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="10"/>
-      <c r="B17" s="33"/>
+      <c r="B17" s="29"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1117,7 +1126,7 @@
       <c r="A18" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="33"/>
+      <c r="B18" s="29"/>
       <c r="C18" s="22">
         <f>SUM(C13:C17)</f>
         <v>12</v>
@@ -1129,7 +1138,7 @@
       <c r="A19" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="34"/>
+      <c r="B19" s="30"/>
       <c r="C19" s="25"/>
       <c r="D19" s="26"/>
       <c r="E19" s="27"/>
@@ -1138,7 +1147,7 @@
       <c r="A20" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B20" s="32">
+      <c r="B20" s="28">
         <v>46050</v>
       </c>
       <c r="C20" s="5">
@@ -1153,7 +1162,7 @@
       <c r="A21" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="33"/>
+      <c r="B21" s="29"/>
       <c r="C21" s="8">
         <v>3</v>
       </c>
@@ -1164,7 +1173,7 @@
     </row>
     <row r="22" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
-      <c r="B22" s="33"/>
+      <c r="B22" s="29"/>
       <c r="C22" s="8">
         <v>2</v>
       </c>
@@ -1175,7 +1184,7 @@
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
-      <c r="B23" s="33"/>
+      <c r="B23" s="29"/>
       <c r="C23" s="8">
         <v>2</v>
       </c>
@@ -1186,7 +1195,7 @@
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="10"/>
-      <c r="B24" s="33"/>
+      <c r="B24" s="29"/>
       <c r="C24" s="10"/>
       <c r="D24" s="11"/>
       <c r="E24" s="10"/>
@@ -1195,7 +1204,7 @@
       <c r="A25" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="33"/>
+      <c r="B25" s="29"/>
       <c r="C25" s="22">
         <f>SUM(C20:C24)</f>
         <v>12</v>
@@ -1207,16 +1216,16 @@
       <c r="A26" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="34"/>
+      <c r="B26" s="30"/>
       <c r="C26" s="25"/>
       <c r="D26" s="26"/>
       <c r="E26" s="27"/>
     </row>
-    <row r="27" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="32">
+      <c r="B27" s="28">
         <v>46057</v>
       </c>
       <c r="C27" s="5">
@@ -1227,9 +1236,11 @@
       </c>
       <c r="E27" s="21"/>
     </row>
-    <row r="28" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="7"/>
-      <c r="B28" s="33"/>
+    <row r="28" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="29"/>
       <c r="C28" s="8">
         <v>3</v>
       </c>
@@ -1239,8 +1250,10 @@
       <c r="E28" s="8"/>
     </row>
     <row r="29" spans="1:5" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="7"/>
-      <c r="B29" s="33"/>
+      <c r="A29" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" s="29"/>
       <c r="C29" s="8">
         <v>4</v>
       </c>
@@ -1251,14 +1264,14 @@
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
-      <c r="B30" s="33"/>
+      <c r="B30" s="29"/>
       <c r="C30" s="8"/>
       <c r="D30" s="9"/>
       <c r="E30" s="8"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="10"/>
-      <c r="B31" s="33"/>
+      <c r="B31" s="29"/>
       <c r="C31" s="10">
         <v>3</v>
       </c>
@@ -1271,7 +1284,7 @@
       <c r="A32" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B32" s="33"/>
+      <c r="B32" s="29"/>
       <c r="C32" s="22">
         <f>SUM(C27:C31)</f>
         <v>12</v>
@@ -1283,55 +1296,63 @@
       <c r="A33" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B33" s="34"/>
+      <c r="B33" s="30"/>
       <c r="C33" s="25"/>
       <c r="D33" s="26"/>
       <c r="E33" s="27"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B34" s="32"/>
+        <v>30</v>
+      </c>
+      <c r="B34" s="28">
+        <v>46062</v>
+      </c>
       <c r="C34" s="5">
-        <v>1</v>
-      </c>
-      <c r="D34" s="6"/>
+        <v>3</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>46</v>
+      </c>
       <c r="E34" s="21"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="7"/>
-      <c r="B35" s="33"/>
+      <c r="A35" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B35" s="29"/>
       <c r="C35" s="8">
-        <v>1</v>
-      </c>
-      <c r="D35" s="9"/>
+        <v>5</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>47</v>
+      </c>
       <c r="E35" s="8"/>
     </row>
-    <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="7"/>
-      <c r="B36" s="33"/>
+    <row r="36" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B36" s="29"/>
       <c r="C36" s="8">
-        <v>1</v>
-      </c>
-      <c r="D36" s="9"/>
+        <v>4</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>48</v>
+      </c>
       <c r="E36" s="8"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
-      <c r="B37" s="33"/>
-      <c r="C37" s="8">
-        <v>1</v>
-      </c>
+      <c r="B37" s="29"/>
+      <c r="C37" s="8"/>
       <c r="D37" s="9"/>
       <c r="E37" s="8"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="10"/>
-      <c r="B38" s="33"/>
-      <c r="C38" s="10">
-        <v>1</v>
-      </c>
+      <c r="B38" s="29"/>
+      <c r="C38" s="10"/>
       <c r="D38" s="11"/>
       <c r="E38" s="10"/>
     </row>
@@ -1339,10 +1360,10 @@
       <c r="A39" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B39" s="33"/>
+      <c r="B39" s="29"/>
       <c r="C39" s="22">
         <f>SUM(C34:C38)</f>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D39" s="23"/>
       <c r="E39" s="24"/>
@@ -1351,7 +1372,7 @@
       <c r="A40" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="34"/>
+      <c r="B40" s="30"/>
       <c r="C40" s="25"/>
       <c r="D40" s="26"/>
       <c r="E40" s="27"/>
@@ -1360,7 +1381,7 @@
       <c r="A41" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B41" s="32"/>
+      <c r="B41" s="28"/>
       <c r="C41" s="5">
         <v>1</v>
       </c>
@@ -1369,7 +1390,7 @@
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="7"/>
-      <c r="B42" s="33"/>
+      <c r="B42" s="29"/>
       <c r="C42" s="8">
         <v>1</v>
       </c>
@@ -1378,7 +1399,7 @@
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7"/>
-      <c r="B43" s="33"/>
+      <c r="B43" s="29"/>
       <c r="C43" s="8">
         <v>1</v>
       </c>
@@ -1387,7 +1408,7 @@
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="7"/>
-      <c r="B44" s="33"/>
+      <c r="B44" s="29"/>
       <c r="C44" s="8">
         <v>1</v>
       </c>
@@ -1396,7 +1417,7 @@
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="10"/>
-      <c r="B45" s="33"/>
+      <c r="B45" s="29"/>
       <c r="C45" s="10">
         <v>1</v>
       </c>
@@ -1407,7 +1428,7 @@
       <c r="A46" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B46" s="33"/>
+      <c r="B46" s="29"/>
       <c r="C46" s="22">
         <f>SUM(C41:C45)</f>
         <v>5</v>
@@ -1419,7 +1440,7 @@
       <c r="A47" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B47" s="34"/>
+      <c r="B47" s="30"/>
       <c r="C47" s="25"/>
       <c r="D47" s="26"/>
       <c r="E47" s="27"/>
@@ -1428,7 +1449,7 @@
       <c r="A48" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="32"/>
+      <c r="B48" s="28"/>
       <c r="C48" s="5">
         <v>1</v>
       </c>
@@ -1437,7 +1458,7 @@
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
-      <c r="B49" s="33"/>
+      <c r="B49" s="29"/>
       <c r="C49" s="8">
         <v>1</v>
       </c>
@@ -1446,7 +1467,7 @@
     </row>
     <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
-      <c r="B50" s="33"/>
+      <c r="B50" s="29"/>
       <c r="C50" s="8">
         <v>1</v>
       </c>
@@ -1455,7 +1476,7 @@
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="7"/>
-      <c r="B51" s="33"/>
+      <c r="B51" s="29"/>
       <c r="C51" s="8">
         <v>1</v>
       </c>
@@ -1464,7 +1485,7 @@
     </row>
     <row r="52" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="10"/>
-      <c r="B52" s="33"/>
+      <c r="B52" s="29"/>
       <c r="C52" s="10">
         <v>1</v>
       </c>
@@ -1475,7 +1496,7 @@
       <c r="A53" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B53" s="33"/>
+      <c r="B53" s="29"/>
       <c r="C53" s="22">
         <f>SUM(C48:C52)</f>
         <v>5</v>
@@ -1487,7 +1508,7 @@
       <c r="A54" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B54" s="34"/>
+      <c r="B54" s="30"/>
       <c r="C54" s="25"/>
       <c r="D54" s="26"/>
       <c r="E54" s="27"/>
@@ -1496,7 +1517,7 @@
       <c r="A55" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B55" s="32"/>
+      <c r="B55" s="28"/>
       <c r="C55" s="5">
         <v>1</v>
       </c>
@@ -1505,7 +1526,7 @@
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="7"/>
-      <c r="B56" s="33"/>
+      <c r="B56" s="29"/>
       <c r="C56" s="8">
         <v>1</v>
       </c>
@@ -1514,7 +1535,7 @@
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="7"/>
-      <c r="B57" s="33"/>
+      <c r="B57" s="29"/>
       <c r="C57" s="8">
         <v>1</v>
       </c>
@@ -1523,7 +1544,7 @@
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="33"/>
+      <c r="B58" s="29"/>
       <c r="C58" s="8">
         <v>1</v>
       </c>
@@ -1532,7 +1553,7 @@
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="10"/>
-      <c r="B59" s="33"/>
+      <c r="B59" s="29"/>
       <c r="C59" s="10">
         <v>1</v>
       </c>
@@ -1543,7 +1564,7 @@
       <c r="A60" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B60" s="33"/>
+      <c r="B60" s="29"/>
       <c r="C60" s="22">
         <f>SUM(C55:C59)</f>
         <v>5</v>
@@ -1555,7 +1576,7 @@
       <c r="A61" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B61" s="34"/>
+      <c r="B61" s="30"/>
       <c r="C61" s="25"/>
       <c r="D61" s="26"/>
       <c r="E61" s="27"/>
@@ -1564,7 +1585,7 @@
       <c r="A62" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B62" s="32"/>
+      <c r="B62" s="28"/>
       <c r="C62" s="5">
         <v>1</v>
       </c>
@@ -1573,7 +1594,7 @@
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
-      <c r="B63" s="33"/>
+      <c r="B63" s="29"/>
       <c r="C63" s="8">
         <v>1</v>
       </c>
@@ -1582,7 +1603,7 @@
     </row>
     <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="33"/>
+      <c r="B64" s="29"/>
       <c r="C64" s="8">
         <v>1</v>
       </c>
@@ -1591,7 +1612,7 @@
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="7"/>
-      <c r="B65" s="33"/>
+      <c r="B65" s="29"/>
       <c r="C65" s="8">
         <v>1</v>
       </c>
@@ -1600,7 +1621,7 @@
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="33"/>
+      <c r="B66" s="29"/>
       <c r="C66" s="10">
         <v>1</v>
       </c>
@@ -1611,7 +1632,7 @@
       <c r="A67" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B67" s="33"/>
+      <c r="B67" s="29"/>
       <c r="C67" s="22">
         <f>SUM(C62:C66)</f>
         <v>5</v>
@@ -1623,7 +1644,7 @@
       <c r="A68" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B68" s="34"/>
+      <c r="B68" s="30"/>
       <c r="C68" s="25"/>
       <c r="D68" s="26"/>
       <c r="E68" s="27"/>
@@ -1632,7 +1653,7 @@
       <c r="A69" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B69" s="32"/>
+      <c r="B69" s="28"/>
       <c r="C69" s="5">
         <v>1</v>
       </c>
@@ -1641,7 +1662,7 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="7"/>
-      <c r="B70" s="33"/>
+      <c r="B70" s="29"/>
       <c r="C70" s="8">
         <v>1</v>
       </c>
@@ -1650,7 +1671,7 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="7"/>
-      <c r="B71" s="33"/>
+      <c r="B71" s="29"/>
       <c r="C71" s="8">
         <v>1</v>
       </c>
@@ -1659,7 +1680,7 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="7"/>
-      <c r="B72" s="33"/>
+      <c r="B72" s="29"/>
       <c r="C72" s="8">
         <v>1</v>
       </c>
@@ -1668,7 +1689,7 @@
     </row>
     <row r="73" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="10"/>
-      <c r="B73" s="33"/>
+      <c r="B73" s="29"/>
       <c r="C73" s="10">
         <v>1</v>
       </c>
@@ -1679,7 +1700,7 @@
       <c r="A74" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B74" s="33"/>
+      <c r="B74" s="29"/>
       <c r="C74" s="22">
         <f>SUM(C69:C73)</f>
         <v>5</v>
@@ -1691,7 +1712,7 @@
       <c r="A75" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B75" s="34"/>
+      <c r="B75" s="30"/>
       <c r="C75" s="25"/>
       <c r="D75" s="26"/>
       <c r="E75" s="27"/>
@@ -1700,7 +1721,7 @@
       <c r="A76" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B76" s="32"/>
+      <c r="B76" s="28"/>
       <c r="C76" s="5">
         <v>1</v>
       </c>
@@ -1709,7 +1730,7 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="7"/>
-      <c r="B77" s="33"/>
+      <c r="B77" s="29"/>
       <c r="C77" s="8">
         <v>1</v>
       </c>
@@ -1718,7 +1739,7 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="7"/>
-      <c r="B78" s="33"/>
+      <c r="B78" s="29"/>
       <c r="C78" s="8">
         <v>1</v>
       </c>
@@ -1727,7 +1748,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="7"/>
-      <c r="B79" s="33"/>
+      <c r="B79" s="29"/>
       <c r="C79" s="8">
         <v>1</v>
       </c>
@@ -1736,7 +1757,7 @@
     </row>
     <row r="80" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="10"/>
-      <c r="B80" s="33"/>
+      <c r="B80" s="29"/>
       <c r="C80" s="10">
         <v>1</v>
       </c>
@@ -1747,7 +1768,7 @@
       <c r="A81" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B81" s="33"/>
+      <c r="B81" s="29"/>
       <c r="C81" s="22">
         <f>SUM(C76:C80)</f>
         <v>5</v>
@@ -1759,7 +1780,7 @@
       <c r="A82" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B82" s="34"/>
+      <c r="B82" s="30"/>
       <c r="C82" s="25"/>
       <c r="D82" s="26"/>
       <c r="E82" s="27"/>
@@ -1768,7 +1789,7 @@
       <c r="A83" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B83" s="32"/>
+      <c r="B83" s="28"/>
       <c r="C83" s="5">
         <v>1</v>
       </c>
@@ -1777,7 +1798,7 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="7"/>
-      <c r="B84" s="33"/>
+      <c r="B84" s="29"/>
       <c r="C84" s="8">
         <v>1</v>
       </c>
@@ -1786,7 +1807,7 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="7"/>
-      <c r="B85" s="33"/>
+      <c r="B85" s="29"/>
       <c r="C85" s="8">
         <v>1</v>
       </c>
@@ -1795,7 +1816,7 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="7"/>
-      <c r="B86" s="33"/>
+      <c r="B86" s="29"/>
       <c r="C86" s="8">
         <v>1</v>
       </c>
@@ -1804,7 +1825,7 @@
     </row>
     <row r="87" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="10"/>
-      <c r="B87" s="33"/>
+      <c r="B87" s="29"/>
       <c r="C87" s="10">
         <v>1</v>
       </c>
@@ -1815,7 +1836,7 @@
       <c r="A88" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B88" s="33"/>
+      <c r="B88" s="29"/>
       <c r="C88" s="22">
         <f>SUM(C83:C87)</f>
         <v>5</v>
@@ -1827,19 +1848,19 @@
       <c r="A89" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B89" s="34"/>
+      <c r="B89" s="30"/>
       <c r="C89" s="25"/>
       <c r="D89" s="26"/>
       <c r="E89" s="27"/>
     </row>
     <row r="90" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="35" t="s">
+      <c r="A90" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="B90" s="36"/>
+      <c r="B90" s="32"/>
       <c r="C90" s="13">
         <f>MROUND(SUM(C6:C89) /8,0.2)</f>
-        <v>22</v>
+        <v>23.8</v>
       </c>
       <c r="D90" s="14"/>
       <c r="E90" s="15"/>
@@ -1854,31 +1875,6 @@
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="D81:E81"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="B83:B89"/>
-    <mergeCell ref="D88:E88"/>
-    <mergeCell ref="C89:E89"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="B69:B75"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="C75:E75"/>
-    <mergeCell ref="B27:B33"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="A90:B90"/>
-    <mergeCell ref="B34:B40"/>
-    <mergeCell ref="B41:B47"/>
-    <mergeCell ref="B48:B54"/>
-    <mergeCell ref="B55:B61"/>
-    <mergeCell ref="B62:B68"/>
-    <mergeCell ref="B76:B82"/>
     <mergeCell ref="D60:E60"/>
     <mergeCell ref="C61:E61"/>
     <mergeCell ref="B1:C1"/>
@@ -1895,6 +1891,31 @@
     <mergeCell ref="B20:B26"/>
     <mergeCell ref="D25:E25"/>
     <mergeCell ref="C26:E26"/>
+    <mergeCell ref="A90:B90"/>
+    <mergeCell ref="B34:B40"/>
+    <mergeCell ref="B41:B47"/>
+    <mergeCell ref="B48:B54"/>
+    <mergeCell ref="B55:B61"/>
+    <mergeCell ref="B62:B68"/>
+    <mergeCell ref="B76:B82"/>
+    <mergeCell ref="B27:B33"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="C47:E47"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="B69:B75"/>
+    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="C75:E75"/>
+    <mergeCell ref="D81:E81"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="B83:B89"/>
+    <mergeCell ref="D88:E88"/>
+    <mergeCell ref="C89:E89"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C11 B13 C13:C18 B20 C20:C25 B27 C27:C32 B34 C34:C39 B41 C41:C46 B48 C48:C53 B55 C55:C60 B62 C62:C67 B69 C69:C74 B76 C76:C81 B83 C83:C88" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -1903,7 +1924,7 @@
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="47" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="46" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -1913,18 +1934,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2090,18 +2111,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
feat(amelioration du recu): amelioration du recu, ajout d'un tableau
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-RayanSahbani-jnltrav.xlsx
+++ b/doc/P-P_OO-RayanSahbani-jnltrav.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML FID1\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{074084A4-7BFF-4A42-81C0-E7641A54EE03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AACA78FF-6993-44F1-AFA8-3EEEEACF0AEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="52">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -197,6 +197,15 @@
   </si>
   <si>
     <t>J'ai amélioré le visuel de mon code et j'ai aussi fais des tests pour voir si tout fonctionne bien.</t>
+  </si>
+  <si>
+    <t>J'ai amélioré le retrait car j'avais des problèmes avec le recu et mon retrait</t>
+  </si>
+  <si>
+    <t>J'ai amélioré mon recu pour qu'il affiche toutes les transactions effectuer alors qu'avant ca affichait que la dernière.</t>
+  </si>
+  <si>
+    <t>J'ai fais ma release et j'ai revisé le test de jeudi</t>
   </si>
 </sst>
 </file>
@@ -541,6 +550,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -558,18 +579,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -904,10 +913,10 @@
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="33"/>
+      <c r="C1" s="28"/>
       <c r="D1" s="20" t="s">
         <v>1</v>
       </c>
@@ -919,10 +928,10 @@
       <c r="A2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="33"/>
+      <c r="C2" s="28"/>
       <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
@@ -934,10 +943,10 @@
       <c r="A3" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="33"/>
+      <c r="C3" s="28"/>
       <c r="D3" s="20" t="s">
         <v>6</v>
       </c>
@@ -949,12 +958,12 @@
       <c r="A4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="36"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="31"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -977,7 +986,7 @@
       <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="28">
+      <c r="B6" s="32">
         <v>46036</v>
       </c>
       <c r="C6" s="5">
@@ -992,7 +1001,7 @@
       <c r="A7" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="29"/>
+      <c r="B7" s="33"/>
       <c r="C7" s="8">
         <v>3</v>
       </c>
@@ -1005,7 +1014,7 @@
       <c r="A8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="29"/>
+      <c r="B8" s="33"/>
       <c r="C8" s="8">
         <v>1</v>
       </c>
@@ -1018,7 +1027,7 @@
       <c r="A9" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="29"/>
+      <c r="B9" s="33"/>
       <c r="C9" s="8">
         <v>2</v>
       </c>
@@ -1031,7 +1040,7 @@
       <c r="A10" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="29"/>
+      <c r="B10" s="33"/>
       <c r="C10" s="10">
         <v>3</v>
       </c>
@@ -1044,7 +1053,7 @@
       <c r="A11" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="29"/>
+      <c r="B11" s="33"/>
       <c r="C11" s="22">
         <f>SUM(C6:C10)</f>
         <v>12</v>
@@ -1056,7 +1065,7 @@
       <c r="A12" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="30"/>
+      <c r="B12" s="34"/>
       <c r="C12" s="25"/>
       <c r="D12" s="26"/>
       <c r="E12" s="27"/>
@@ -1065,7 +1074,7 @@
       <c r="A13" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="28">
+      <c r="B13" s="32">
         <v>46043</v>
       </c>
       <c r="C13" s="5">
@@ -1080,7 +1089,7 @@
       <c r="A14" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="29"/>
+      <c r="B14" s="33"/>
       <c r="C14" s="8">
         <v>5</v>
       </c>
@@ -1093,7 +1102,7 @@
       <c r="A15" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="29"/>
+      <c r="B15" s="33"/>
       <c r="C15" s="8">
         <v>4</v>
       </c>
@@ -1106,7 +1115,7 @@
       <c r="A16" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="29"/>
+      <c r="B16" s="33"/>
       <c r="C16" s="8">
         <v>1</v>
       </c>
@@ -1117,7 +1126,7 @@
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="10"/>
-      <c r="B17" s="29"/>
+      <c r="B17" s="33"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1126,7 +1135,7 @@
       <c r="A18" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="29"/>
+      <c r="B18" s="33"/>
       <c r="C18" s="22">
         <f>SUM(C13:C17)</f>
         <v>12</v>
@@ -1138,7 +1147,7 @@
       <c r="A19" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="30"/>
+      <c r="B19" s="34"/>
       <c r="C19" s="25"/>
       <c r="D19" s="26"/>
       <c r="E19" s="27"/>
@@ -1147,7 +1156,7 @@
       <c r="A20" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B20" s="28">
+      <c r="B20" s="32">
         <v>46050</v>
       </c>
       <c r="C20" s="5">
@@ -1162,7 +1171,7 @@
       <c r="A21" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="29"/>
+      <c r="B21" s="33"/>
       <c r="C21" s="8">
         <v>3</v>
       </c>
@@ -1173,7 +1182,7 @@
     </row>
     <row r="22" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
-      <c r="B22" s="29"/>
+      <c r="B22" s="33"/>
       <c r="C22" s="8">
         <v>2</v>
       </c>
@@ -1184,7 +1193,7 @@
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
-      <c r="B23" s="29"/>
+      <c r="B23" s="33"/>
       <c r="C23" s="8">
         <v>2</v>
       </c>
@@ -1195,7 +1204,7 @@
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="10"/>
-      <c r="B24" s="29"/>
+      <c r="B24" s="33"/>
       <c r="C24" s="10"/>
       <c r="D24" s="11"/>
       <c r="E24" s="10"/>
@@ -1204,7 +1213,7 @@
       <c r="A25" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="29"/>
+      <c r="B25" s="33"/>
       <c r="C25" s="22">
         <f>SUM(C20:C24)</f>
         <v>12</v>
@@ -1216,7 +1225,7 @@
       <c r="A26" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="30"/>
+      <c r="B26" s="34"/>
       <c r="C26" s="25"/>
       <c r="D26" s="26"/>
       <c r="E26" s="27"/>
@@ -1225,7 +1234,7 @@
       <c r="A27" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="28">
+      <c r="B27" s="32">
         <v>46057</v>
       </c>
       <c r="C27" s="5">
@@ -1240,7 +1249,7 @@
       <c r="A28" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B28" s="29"/>
+      <c r="B28" s="33"/>
       <c r="C28" s="8">
         <v>3</v>
       </c>
@@ -1253,7 +1262,7 @@
       <c r="A29" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="29"/>
+      <c r="B29" s="33"/>
       <c r="C29" s="8">
         <v>4</v>
       </c>
@@ -1264,14 +1273,14 @@
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
-      <c r="B30" s="29"/>
+      <c r="B30" s="33"/>
       <c r="C30" s="8"/>
       <c r="D30" s="9"/>
       <c r="E30" s="8"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="10"/>
-      <c r="B31" s="29"/>
+      <c r="B31" s="33"/>
       <c r="C31" s="10">
         <v>3</v>
       </c>
@@ -1284,7 +1293,7 @@
       <c r="A32" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B32" s="29"/>
+      <c r="B32" s="33"/>
       <c r="C32" s="22">
         <f>SUM(C27:C31)</f>
         <v>12</v>
@@ -1296,7 +1305,7 @@
       <c r="A33" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B33" s="30"/>
+      <c r="B33" s="34"/>
       <c r="C33" s="25"/>
       <c r="D33" s="26"/>
       <c r="E33" s="27"/>
@@ -1305,7 +1314,7 @@
       <c r="A34" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B34" s="28">
+      <c r="B34" s="32">
         <v>46062</v>
       </c>
       <c r="C34" s="5">
@@ -1320,7 +1329,7 @@
       <c r="A35" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B35" s="29"/>
+      <c r="B35" s="33"/>
       <c r="C35" s="8">
         <v>5</v>
       </c>
@@ -1333,7 +1342,7 @@
       <c r="A36" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B36" s="29"/>
+      <c r="B36" s="33"/>
       <c r="C36" s="8">
         <v>4</v>
       </c>
@@ -1344,14 +1353,14 @@
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
-      <c r="B37" s="29"/>
+      <c r="B37" s="33"/>
       <c r="C37" s="8"/>
       <c r="D37" s="9"/>
       <c r="E37" s="8"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="10"/>
-      <c r="B38" s="29"/>
+      <c r="B38" s="33"/>
       <c r="C38" s="10"/>
       <c r="D38" s="11"/>
       <c r="E38" s="10"/>
@@ -1360,7 +1369,7 @@
       <c r="A39" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B39" s="29"/>
+      <c r="B39" s="33"/>
       <c r="C39" s="22">
         <f>SUM(C34:C38)</f>
         <v>12</v>
@@ -1372,55 +1381,61 @@
       <c r="A40" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="30"/>
+      <c r="B40" s="34"/>
       <c r="C40" s="25"/>
       <c r="D40" s="26"/>
       <c r="E40" s="27"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B41" s="28"/>
+        <v>30</v>
+      </c>
+      <c r="B41" s="32">
+        <v>46064</v>
+      </c>
       <c r="C41" s="5">
-        <v>1</v>
-      </c>
-      <c r="D41" s="6"/>
+        <v>3</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>49</v>
+      </c>
       <c r="E41" s="21"/>
     </row>
-    <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="7"/>
-      <c r="B42" s="29"/>
+    <row r="42" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A42" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B42" s="33"/>
       <c r="C42" s="8">
-        <v>1</v>
-      </c>
-      <c r="D42" s="9"/>
+        <v>4</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>50</v>
+      </c>
       <c r="E42" s="8"/>
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7"/>
-      <c r="B43" s="29"/>
+      <c r="B43" s="33"/>
       <c r="C43" s="8">
-        <v>1</v>
-      </c>
-      <c r="D43" s="9"/>
+        <v>5</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>51</v>
+      </c>
       <c r="E43" s="8"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="7"/>
-      <c r="B44" s="29"/>
-      <c r="C44" s="8">
-        <v>1</v>
-      </c>
+      <c r="B44" s="33"/>
+      <c r="C44" s="8"/>
       <c r="D44" s="9"/>
       <c r="E44" s="8"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="10"/>
-      <c r="B45" s="29"/>
-      <c r="C45" s="10">
-        <v>1</v>
-      </c>
+      <c r="B45" s="33"/>
+      <c r="C45" s="10"/>
       <c r="D45" s="11"/>
       <c r="E45" s="10"/>
     </row>
@@ -1428,10 +1443,10 @@
       <c r="A46" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B46" s="29"/>
+      <c r="B46" s="33"/>
       <c r="C46" s="22">
         <f>SUM(C41:C45)</f>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D46" s="23"/>
       <c r="E46" s="24"/>
@@ -1440,7 +1455,7 @@
       <c r="A47" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B47" s="30"/>
+      <c r="B47" s="34"/>
       <c r="C47" s="25"/>
       <c r="D47" s="26"/>
       <c r="E47" s="27"/>
@@ -1449,7 +1464,7 @@
       <c r="A48" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B48" s="28"/>
+      <c r="B48" s="32"/>
       <c r="C48" s="5">
         <v>1</v>
       </c>
@@ -1458,7 +1473,7 @@
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
-      <c r="B49" s="29"/>
+      <c r="B49" s="33"/>
       <c r="C49" s="8">
         <v>1</v>
       </c>
@@ -1467,7 +1482,7 @@
     </row>
     <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
-      <c r="B50" s="29"/>
+      <c r="B50" s="33"/>
       <c r="C50" s="8">
         <v>1</v>
       </c>
@@ -1476,7 +1491,7 @@
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="7"/>
-      <c r="B51" s="29"/>
+      <c r="B51" s="33"/>
       <c r="C51" s="8">
         <v>1</v>
       </c>
@@ -1485,7 +1500,7 @@
     </row>
     <row r="52" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="10"/>
-      <c r="B52" s="29"/>
+      <c r="B52" s="33"/>
       <c r="C52" s="10">
         <v>1</v>
       </c>
@@ -1496,7 +1511,7 @@
       <c r="A53" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B53" s="29"/>
+      <c r="B53" s="33"/>
       <c r="C53" s="22">
         <f>SUM(C48:C52)</f>
         <v>5</v>
@@ -1508,7 +1523,7 @@
       <c r="A54" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B54" s="30"/>
+      <c r="B54" s="34"/>
       <c r="C54" s="25"/>
       <c r="D54" s="26"/>
       <c r="E54" s="27"/>
@@ -1517,7 +1532,7 @@
       <c r="A55" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B55" s="28"/>
+      <c r="B55" s="32"/>
       <c r="C55" s="5">
         <v>1</v>
       </c>
@@ -1526,7 +1541,7 @@
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="7"/>
-      <c r="B56" s="29"/>
+      <c r="B56" s="33"/>
       <c r="C56" s="8">
         <v>1</v>
       </c>
@@ -1535,7 +1550,7 @@
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="7"/>
-      <c r="B57" s="29"/>
+      <c r="B57" s="33"/>
       <c r="C57" s="8">
         <v>1</v>
       </c>
@@ -1544,7 +1559,7 @@
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="29"/>
+      <c r="B58" s="33"/>
       <c r="C58" s="8">
         <v>1</v>
       </c>
@@ -1553,7 +1568,7 @@
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="10"/>
-      <c r="B59" s="29"/>
+      <c r="B59" s="33"/>
       <c r="C59" s="10">
         <v>1</v>
       </c>
@@ -1564,7 +1579,7 @@
       <c r="A60" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B60" s="29"/>
+      <c r="B60" s="33"/>
       <c r="C60" s="22">
         <f>SUM(C55:C59)</f>
         <v>5</v>
@@ -1576,7 +1591,7 @@
       <c r="A61" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B61" s="30"/>
+      <c r="B61" s="34"/>
       <c r="C61" s="25"/>
       <c r="D61" s="26"/>
       <c r="E61" s="27"/>
@@ -1585,7 +1600,7 @@
       <c r="A62" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B62" s="28"/>
+      <c r="B62" s="32"/>
       <c r="C62" s="5">
         <v>1</v>
       </c>
@@ -1594,7 +1609,7 @@
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
-      <c r="B63" s="29"/>
+      <c r="B63" s="33"/>
       <c r="C63" s="8">
         <v>1</v>
       </c>
@@ -1603,7 +1618,7 @@
     </row>
     <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="29"/>
+      <c r="B64" s="33"/>
       <c r="C64" s="8">
         <v>1</v>
       </c>
@@ -1612,7 +1627,7 @@
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="7"/>
-      <c r="B65" s="29"/>
+      <c r="B65" s="33"/>
       <c r="C65" s="8">
         <v>1</v>
       </c>
@@ -1621,7 +1636,7 @@
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="29"/>
+      <c r="B66" s="33"/>
       <c r="C66" s="10">
         <v>1</v>
       </c>
@@ -1632,7 +1647,7 @@
       <c r="A67" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B67" s="29"/>
+      <c r="B67" s="33"/>
       <c r="C67" s="22">
         <f>SUM(C62:C66)</f>
         <v>5</v>
@@ -1644,7 +1659,7 @@
       <c r="A68" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B68" s="30"/>
+      <c r="B68" s="34"/>
       <c r="C68" s="25"/>
       <c r="D68" s="26"/>
       <c r="E68" s="27"/>
@@ -1653,7 +1668,7 @@
       <c r="A69" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B69" s="28"/>
+      <c r="B69" s="32"/>
       <c r="C69" s="5">
         <v>1</v>
       </c>
@@ -1662,7 +1677,7 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="7"/>
-      <c r="B70" s="29"/>
+      <c r="B70" s="33"/>
       <c r="C70" s="8">
         <v>1</v>
       </c>
@@ -1671,7 +1686,7 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="7"/>
-      <c r="B71" s="29"/>
+      <c r="B71" s="33"/>
       <c r="C71" s="8">
         <v>1</v>
       </c>
@@ -1680,7 +1695,7 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="7"/>
-      <c r="B72" s="29"/>
+      <c r="B72" s="33"/>
       <c r="C72" s="8">
         <v>1</v>
       </c>
@@ -1689,7 +1704,7 @@
     </row>
     <row r="73" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="10"/>
-      <c r="B73" s="29"/>
+      <c r="B73" s="33"/>
       <c r="C73" s="10">
         <v>1</v>
       </c>
@@ -1700,7 +1715,7 @@
       <c r="A74" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B74" s="29"/>
+      <c r="B74" s="33"/>
       <c r="C74" s="22">
         <f>SUM(C69:C73)</f>
         <v>5</v>
@@ -1712,7 +1727,7 @@
       <c r="A75" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B75" s="30"/>
+      <c r="B75" s="34"/>
       <c r="C75" s="25"/>
       <c r="D75" s="26"/>
       <c r="E75" s="27"/>
@@ -1721,7 +1736,7 @@
       <c r="A76" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B76" s="28"/>
+      <c r="B76" s="32"/>
       <c r="C76" s="5">
         <v>1</v>
       </c>
@@ -1730,7 +1745,7 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="7"/>
-      <c r="B77" s="29"/>
+      <c r="B77" s="33"/>
       <c r="C77" s="8">
         <v>1</v>
       </c>
@@ -1739,7 +1754,7 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="7"/>
-      <c r="B78" s="29"/>
+      <c r="B78" s="33"/>
       <c r="C78" s="8">
         <v>1</v>
       </c>
@@ -1748,7 +1763,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="7"/>
-      <c r="B79" s="29"/>
+      <c r="B79" s="33"/>
       <c r="C79" s="8">
         <v>1</v>
       </c>
@@ -1757,7 +1772,7 @@
     </row>
     <row r="80" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="10"/>
-      <c r="B80" s="29"/>
+      <c r="B80" s="33"/>
       <c r="C80" s="10">
         <v>1</v>
       </c>
@@ -1768,7 +1783,7 @@
       <c r="A81" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B81" s="29"/>
+      <c r="B81" s="33"/>
       <c r="C81" s="22">
         <f>SUM(C76:C80)</f>
         <v>5</v>
@@ -1780,7 +1795,7 @@
       <c r="A82" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B82" s="30"/>
+      <c r="B82" s="34"/>
       <c r="C82" s="25"/>
       <c r="D82" s="26"/>
       <c r="E82" s="27"/>
@@ -1789,7 +1804,7 @@
       <c r="A83" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B83" s="28"/>
+      <c r="B83" s="32"/>
       <c r="C83" s="5">
         <v>1</v>
       </c>
@@ -1798,7 +1813,7 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="7"/>
-      <c r="B84" s="29"/>
+      <c r="B84" s="33"/>
       <c r="C84" s="8">
         <v>1</v>
       </c>
@@ -1807,7 +1822,7 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="7"/>
-      <c r="B85" s="29"/>
+      <c r="B85" s="33"/>
       <c r="C85" s="8">
         <v>1</v>
       </c>
@@ -1816,7 +1831,7 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="7"/>
-      <c r="B86" s="29"/>
+      <c r="B86" s="33"/>
       <c r="C86" s="8">
         <v>1</v>
       </c>
@@ -1825,7 +1840,7 @@
     </row>
     <row r="87" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="10"/>
-      <c r="B87" s="29"/>
+      <c r="B87" s="33"/>
       <c r="C87" s="10">
         <v>1</v>
       </c>
@@ -1836,7 +1851,7 @@
       <c r="A88" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B88" s="29"/>
+      <c r="B88" s="33"/>
       <c r="C88" s="22">
         <f>SUM(C83:C87)</f>
         <v>5</v>
@@ -1848,19 +1863,19 @@
       <c r="A89" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B89" s="30"/>
+      <c r="B89" s="34"/>
       <c r="C89" s="25"/>
       <c r="D89" s="26"/>
       <c r="E89" s="27"/>
     </row>
     <row r="90" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="31" t="s">
+      <c r="A90" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="B90" s="32"/>
+      <c r="B90" s="36"/>
       <c r="C90" s="13">
         <f>MROUND(SUM(C6:C89) /8,0.2)</f>
-        <v>23.8</v>
+        <v>25.6</v>
       </c>
       <c r="D90" s="14"/>
       <c r="E90" s="15"/>
@@ -1875,6 +1890,31 @@
     </row>
   </sheetData>
   <mergeCells count="41">
+    <mergeCell ref="D81:E81"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="B83:B89"/>
+    <mergeCell ref="D88:E88"/>
+    <mergeCell ref="C89:E89"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="B69:B75"/>
+    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="C75:E75"/>
+    <mergeCell ref="B27:B33"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="C47:E47"/>
+    <mergeCell ref="A90:B90"/>
+    <mergeCell ref="B34:B40"/>
+    <mergeCell ref="B41:B47"/>
+    <mergeCell ref="B48:B54"/>
+    <mergeCell ref="B55:B61"/>
+    <mergeCell ref="B62:B68"/>
+    <mergeCell ref="B76:B82"/>
     <mergeCell ref="D60:E60"/>
     <mergeCell ref="C61:E61"/>
     <mergeCell ref="B1:C1"/>
@@ -1891,31 +1931,6 @@
     <mergeCell ref="B20:B26"/>
     <mergeCell ref="D25:E25"/>
     <mergeCell ref="C26:E26"/>
-    <mergeCell ref="A90:B90"/>
-    <mergeCell ref="B34:B40"/>
-    <mergeCell ref="B41:B47"/>
-    <mergeCell ref="B48:B54"/>
-    <mergeCell ref="B55:B61"/>
-    <mergeCell ref="B62:B68"/>
-    <mergeCell ref="B76:B82"/>
-    <mergeCell ref="B27:B33"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="B69:B75"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="C75:E75"/>
-    <mergeCell ref="D81:E81"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="B83:B89"/>
-    <mergeCell ref="D88:E88"/>
-    <mergeCell ref="C89:E89"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C11 B13 C13:C18 B20 C20:C25 B27 C27:C32 B34 C34:C39 B41 C41:C46 B48 C48:C53 B55 C55:C60 B62 C62:C67 B69 C69:C74 B76 C76:C81 B83 C83:C88" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -1934,18 +1949,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2111,18 +2126,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
feat(encapsulation et instance): encasuplation et instance terminer et ajout du rapport
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-RayanSahbani-jnltrav.xlsx
+++ b/doc/P-P_OO-RayanSahbani-jnltrav.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML FID1\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AACA78FF-6993-44F1-AFA8-3EEEEACF0AEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4179F20D-2A2D-468F-9909-58337BDE5DA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="56">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -206,6 +206,18 @@
   </si>
   <si>
     <t>J'ai fais ma release et j'ai revisé le test de jeudi</t>
+  </si>
+  <si>
+    <t>J'ai ajouté mon rapport dans la branche et j'ai fais des changements sur mon code ajout des entetes….</t>
+  </si>
+  <si>
+    <t>J'ai fais les instances</t>
+  </si>
+  <si>
+    <t>J'ai eu un probleme avec certaines de mes fonctions qui ma pris du temps</t>
+  </si>
+  <si>
+    <t>J'ai fais l'encapsulation.</t>
   </si>
 </sst>
 </file>
@@ -550,18 +562,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -579,6 +579,18 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -913,10 +925,10 @@
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="28"/>
+      <c r="C1" s="33"/>
       <c r="D1" s="20" t="s">
         <v>1</v>
       </c>
@@ -928,10 +940,10 @@
       <c r="A2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="28"/>
+      <c r="C2" s="33"/>
       <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
@@ -943,10 +955,10 @@
       <c r="A3" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="28"/>
+      <c r="C3" s="33"/>
       <c r="D3" s="20" t="s">
         <v>6</v>
       </c>
@@ -958,12 +970,12 @@
       <c r="A4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="31"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="36"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -986,7 +998,7 @@
       <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="32">
+      <c r="B6" s="28">
         <v>46036</v>
       </c>
       <c r="C6" s="5">
@@ -1001,7 +1013,7 @@
       <c r="A7" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="33"/>
+      <c r="B7" s="29"/>
       <c r="C7" s="8">
         <v>3</v>
       </c>
@@ -1014,7 +1026,7 @@
       <c r="A8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="33"/>
+      <c r="B8" s="29"/>
       <c r="C8" s="8">
         <v>1</v>
       </c>
@@ -1027,7 +1039,7 @@
       <c r="A9" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="33"/>
+      <c r="B9" s="29"/>
       <c r="C9" s="8">
         <v>2</v>
       </c>
@@ -1040,7 +1052,7 @@
       <c r="A10" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="33"/>
+      <c r="B10" s="29"/>
       <c r="C10" s="10">
         <v>3</v>
       </c>
@@ -1053,7 +1065,7 @@
       <c r="A11" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="33"/>
+      <c r="B11" s="29"/>
       <c r="C11" s="22">
         <f>SUM(C6:C10)</f>
         <v>12</v>
@@ -1065,7 +1077,7 @@
       <c r="A12" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="34"/>
+      <c r="B12" s="30"/>
       <c r="C12" s="25"/>
       <c r="D12" s="26"/>
       <c r="E12" s="27"/>
@@ -1074,7 +1086,7 @@
       <c r="A13" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="32">
+      <c r="B13" s="28">
         <v>46043</v>
       </c>
       <c r="C13" s="5">
@@ -1089,7 +1101,7 @@
       <c r="A14" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="33"/>
+      <c r="B14" s="29"/>
       <c r="C14" s="8">
         <v>5</v>
       </c>
@@ -1102,7 +1114,7 @@
       <c r="A15" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="33"/>
+      <c r="B15" s="29"/>
       <c r="C15" s="8">
         <v>4</v>
       </c>
@@ -1115,7 +1127,7 @@
       <c r="A16" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="33"/>
+      <c r="B16" s="29"/>
       <c r="C16" s="8">
         <v>1</v>
       </c>
@@ -1126,7 +1138,7 @@
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="10"/>
-      <c r="B17" s="33"/>
+      <c r="B17" s="29"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1135,7 +1147,7 @@
       <c r="A18" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="33"/>
+      <c r="B18" s="29"/>
       <c r="C18" s="22">
         <f>SUM(C13:C17)</f>
         <v>12</v>
@@ -1147,7 +1159,7 @@
       <c r="A19" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="34"/>
+      <c r="B19" s="30"/>
       <c r="C19" s="25"/>
       <c r="D19" s="26"/>
       <c r="E19" s="27"/>
@@ -1156,7 +1168,7 @@
       <c r="A20" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B20" s="32">
+      <c r="B20" s="28">
         <v>46050</v>
       </c>
       <c r="C20" s="5">
@@ -1171,7 +1183,7 @@
       <c r="A21" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="33"/>
+      <c r="B21" s="29"/>
       <c r="C21" s="8">
         <v>3</v>
       </c>
@@ -1182,7 +1194,7 @@
     </row>
     <row r="22" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
-      <c r="B22" s="33"/>
+      <c r="B22" s="29"/>
       <c r="C22" s="8">
         <v>2</v>
       </c>
@@ -1193,7 +1205,7 @@
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
-      <c r="B23" s="33"/>
+      <c r="B23" s="29"/>
       <c r="C23" s="8">
         <v>2</v>
       </c>
@@ -1204,7 +1216,7 @@
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="10"/>
-      <c r="B24" s="33"/>
+      <c r="B24" s="29"/>
       <c r="C24" s="10"/>
       <c r="D24" s="11"/>
       <c r="E24" s="10"/>
@@ -1213,7 +1225,7 @@
       <c r="A25" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="33"/>
+      <c r="B25" s="29"/>
       <c r="C25" s="22">
         <f>SUM(C20:C24)</f>
         <v>12</v>
@@ -1225,7 +1237,7 @@
       <c r="A26" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="34"/>
+      <c r="B26" s="30"/>
       <c r="C26" s="25"/>
       <c r="D26" s="26"/>
       <c r="E26" s="27"/>
@@ -1234,7 +1246,7 @@
       <c r="A27" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="32">
+      <c r="B27" s="28">
         <v>46057</v>
       </c>
       <c r="C27" s="5">
@@ -1249,7 +1261,7 @@
       <c r="A28" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B28" s="33"/>
+      <c r="B28" s="29"/>
       <c r="C28" s="8">
         <v>3</v>
       </c>
@@ -1262,7 +1274,7 @@
       <c r="A29" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="33"/>
+      <c r="B29" s="29"/>
       <c r="C29" s="8">
         <v>4</v>
       </c>
@@ -1273,14 +1285,14 @@
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
-      <c r="B30" s="33"/>
+      <c r="B30" s="29"/>
       <c r="C30" s="8"/>
       <c r="D30" s="9"/>
       <c r="E30" s="8"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="10"/>
-      <c r="B31" s="33"/>
+      <c r="B31" s="29"/>
       <c r="C31" s="10">
         <v>3</v>
       </c>
@@ -1293,7 +1305,7 @@
       <c r="A32" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B32" s="33"/>
+      <c r="B32" s="29"/>
       <c r="C32" s="22">
         <f>SUM(C27:C31)</f>
         <v>12</v>
@@ -1305,7 +1317,7 @@
       <c r="A33" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B33" s="34"/>
+      <c r="B33" s="30"/>
       <c r="C33" s="25"/>
       <c r="D33" s="26"/>
       <c r="E33" s="27"/>
@@ -1314,7 +1326,7 @@
       <c r="A34" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B34" s="32">
+      <c r="B34" s="28">
         <v>46062</v>
       </c>
       <c r="C34" s="5">
@@ -1329,7 +1341,7 @@
       <c r="A35" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B35" s="33"/>
+      <c r="B35" s="29"/>
       <c r="C35" s="8">
         <v>5</v>
       </c>
@@ -1342,7 +1354,7 @@
       <c r="A36" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B36" s="33"/>
+      <c r="B36" s="29"/>
       <c r="C36" s="8">
         <v>4</v>
       </c>
@@ -1353,14 +1365,14 @@
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
-      <c r="B37" s="33"/>
+      <c r="B37" s="29"/>
       <c r="C37" s="8"/>
       <c r="D37" s="9"/>
       <c r="E37" s="8"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="10"/>
-      <c r="B38" s="33"/>
+      <c r="B38" s="29"/>
       <c r="C38" s="10"/>
       <c r="D38" s="11"/>
       <c r="E38" s="10"/>
@@ -1369,7 +1381,7 @@
       <c r="A39" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B39" s="33"/>
+      <c r="B39" s="29"/>
       <c r="C39" s="22">
         <f>SUM(C34:C38)</f>
         <v>12</v>
@@ -1381,7 +1393,7 @@
       <c r="A40" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="34"/>
+      <c r="B40" s="30"/>
       <c r="C40" s="25"/>
       <c r="D40" s="26"/>
       <c r="E40" s="27"/>
@@ -1390,7 +1402,7 @@
       <c r="A41" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B41" s="32">
+      <c r="B41" s="28">
         <v>46064</v>
       </c>
       <c r="C41" s="5">
@@ -1405,7 +1417,7 @@
       <c r="A42" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B42" s="33"/>
+      <c r="B42" s="29"/>
       <c r="C42" s="8">
         <v>4</v>
       </c>
@@ -1416,7 +1428,7 @@
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7"/>
-      <c r="B43" s="33"/>
+      <c r="B43" s="29"/>
       <c r="C43" s="8">
         <v>5</v>
       </c>
@@ -1427,14 +1439,14 @@
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="7"/>
-      <c r="B44" s="33"/>
+      <c r="B44" s="29"/>
       <c r="C44" s="8"/>
       <c r="D44" s="9"/>
       <c r="E44" s="8"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="10"/>
-      <c r="B45" s="33"/>
+      <c r="B45" s="29"/>
       <c r="C45" s="10"/>
       <c r="D45" s="11"/>
       <c r="E45" s="10"/>
@@ -1443,7 +1455,7 @@
       <c r="A46" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B46" s="33"/>
+      <c r="B46" s="29"/>
       <c r="C46" s="22">
         <f>SUM(C41:C45)</f>
         <v>12</v>
@@ -1455,55 +1467,51 @@
       <c r="A47" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B47" s="34"/>
+      <c r="B47" s="30"/>
       <c r="C47" s="25"/>
       <c r="D47" s="26"/>
       <c r="E47" s="27"/>
     </row>
-    <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B48" s="32"/>
+        <v>30</v>
+      </c>
+      <c r="B48" s="28">
+        <v>46076</v>
+      </c>
       <c r="C48" s="5">
-        <v>1</v>
-      </c>
-      <c r="D48" s="6"/>
+        <v>4</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>52</v>
+      </c>
       <c r="E48" s="21"/>
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
-      <c r="B49" s="33"/>
-      <c r="C49" s="8">
-        <v>1</v>
-      </c>
+      <c r="B49" s="29"/>
+      <c r="C49" s="8"/>
       <c r="D49" s="9"/>
       <c r="E49" s="8"/>
     </row>
     <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
-      <c r="B50" s="33"/>
-      <c r="C50" s="8">
-        <v>1</v>
-      </c>
+      <c r="B50" s="29"/>
+      <c r="C50" s="8"/>
       <c r="D50" s="9"/>
       <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="7"/>
-      <c r="B51" s="33"/>
-      <c r="C51" s="8">
-        <v>1</v>
-      </c>
+      <c r="B51" s="29"/>
+      <c r="C51" s="8"/>
       <c r="D51" s="9"/>
       <c r="E51" s="8"/>
     </row>
     <row r="52" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="10"/>
-      <c r="B52" s="33"/>
-      <c r="C52" s="10">
-        <v>1</v>
-      </c>
+      <c r="B52" s="29"/>
+      <c r="C52" s="10"/>
       <c r="D52" s="11"/>
       <c r="E52" s="10"/>
     </row>
@@ -1511,10 +1519,10 @@
       <c r="A53" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B53" s="33"/>
+      <c r="B53" s="29"/>
       <c r="C53" s="22">
         <f>SUM(C48:C52)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D53" s="23"/>
       <c r="E53" s="24"/>
@@ -1523,55 +1531,63 @@
       <c r="A54" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B54" s="34"/>
+      <c r="B54" s="30"/>
       <c r="C54" s="25"/>
       <c r="D54" s="26"/>
       <c r="E54" s="27"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B55" s="32"/>
+        <v>30</v>
+      </c>
+      <c r="B55" s="28">
+        <v>46078</v>
+      </c>
       <c r="C55" s="5">
-        <v>1</v>
-      </c>
-      <c r="D55" s="6"/>
+        <v>4</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>53</v>
+      </c>
       <c r="E55" s="21"/>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="7"/>
-      <c r="B56" s="33"/>
+      <c r="A56" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B56" s="29"/>
       <c r="C56" s="8">
-        <v>1</v>
-      </c>
-      <c r="D56" s="9"/>
+        <v>4</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>54</v>
+      </c>
       <c r="E56" s="8"/>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="7"/>
-      <c r="B57" s="33"/>
+      <c r="A57" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B57" s="29"/>
       <c r="C57" s="8">
-        <v>1</v>
-      </c>
-      <c r="D57" s="9"/>
+        <v>4</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>55</v>
+      </c>
       <c r="E57" s="8"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="33"/>
-      <c r="C58" s="8">
-        <v>1</v>
-      </c>
+      <c r="B58" s="29"/>
+      <c r="C58" s="8"/>
       <c r="D58" s="9"/>
       <c r="E58" s="8"/>
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="10"/>
-      <c r="B59" s="33"/>
-      <c r="C59" s="10">
-        <v>1</v>
-      </c>
+      <c r="B59" s="29"/>
+      <c r="C59" s="10"/>
       <c r="D59" s="11"/>
       <c r="E59" s="10"/>
     </row>
@@ -1579,10 +1595,10 @@
       <c r="A60" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B60" s="33"/>
+      <c r="B60" s="29"/>
       <c r="C60" s="22">
         <f>SUM(C55:C59)</f>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D60" s="23"/>
       <c r="E60" s="24"/>
@@ -1591,7 +1607,7 @@
       <c r="A61" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B61" s="34"/>
+      <c r="B61" s="30"/>
       <c r="C61" s="25"/>
       <c r="D61" s="26"/>
       <c r="E61" s="27"/>
@@ -1600,7 +1616,7 @@
       <c r="A62" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B62" s="32"/>
+      <c r="B62" s="28"/>
       <c r="C62" s="5">
         <v>1</v>
       </c>
@@ -1609,7 +1625,7 @@
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
-      <c r="B63" s="33"/>
+      <c r="B63" s="29"/>
       <c r="C63" s="8">
         <v>1</v>
       </c>
@@ -1618,7 +1634,7 @@
     </row>
     <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="33"/>
+      <c r="B64" s="29"/>
       <c r="C64" s="8">
         <v>1</v>
       </c>
@@ -1627,7 +1643,7 @@
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="7"/>
-      <c r="B65" s="33"/>
+      <c r="B65" s="29"/>
       <c r="C65" s="8">
         <v>1</v>
       </c>
@@ -1636,7 +1652,7 @@
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="33"/>
+      <c r="B66" s="29"/>
       <c r="C66" s="10">
         <v>1</v>
       </c>
@@ -1647,7 +1663,7 @@
       <c r="A67" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B67" s="33"/>
+      <c r="B67" s="29"/>
       <c r="C67" s="22">
         <f>SUM(C62:C66)</f>
         <v>5</v>
@@ -1659,7 +1675,7 @@
       <c r="A68" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B68" s="34"/>
+      <c r="B68" s="30"/>
       <c r="C68" s="25"/>
       <c r="D68" s="26"/>
       <c r="E68" s="27"/>
@@ -1668,7 +1684,7 @@
       <c r="A69" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B69" s="32"/>
+      <c r="B69" s="28"/>
       <c r="C69" s="5">
         <v>1</v>
       </c>
@@ -1677,7 +1693,7 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="7"/>
-      <c r="B70" s="33"/>
+      <c r="B70" s="29"/>
       <c r="C70" s="8">
         <v>1</v>
       </c>
@@ -1686,7 +1702,7 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="7"/>
-      <c r="B71" s="33"/>
+      <c r="B71" s="29"/>
       <c r="C71" s="8">
         <v>1</v>
       </c>
@@ -1695,7 +1711,7 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="7"/>
-      <c r="B72" s="33"/>
+      <c r="B72" s="29"/>
       <c r="C72" s="8">
         <v>1</v>
       </c>
@@ -1704,7 +1720,7 @@
     </row>
     <row r="73" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="10"/>
-      <c r="B73" s="33"/>
+      <c r="B73" s="29"/>
       <c r="C73" s="10">
         <v>1</v>
       </c>
@@ -1715,7 +1731,7 @@
       <c r="A74" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B74" s="33"/>
+      <c r="B74" s="29"/>
       <c r="C74" s="22">
         <f>SUM(C69:C73)</f>
         <v>5</v>
@@ -1727,7 +1743,7 @@
       <c r="A75" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B75" s="34"/>
+      <c r="B75" s="30"/>
       <c r="C75" s="25"/>
       <c r="D75" s="26"/>
       <c r="E75" s="27"/>
@@ -1736,7 +1752,7 @@
       <c r="A76" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B76" s="32"/>
+      <c r="B76" s="28"/>
       <c r="C76" s="5">
         <v>1</v>
       </c>
@@ -1745,7 +1761,7 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="7"/>
-      <c r="B77" s="33"/>
+      <c r="B77" s="29"/>
       <c r="C77" s="8">
         <v>1</v>
       </c>
@@ -1754,7 +1770,7 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="7"/>
-      <c r="B78" s="33"/>
+      <c r="B78" s="29"/>
       <c r="C78" s="8">
         <v>1</v>
       </c>
@@ -1763,7 +1779,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="7"/>
-      <c r="B79" s="33"/>
+      <c r="B79" s="29"/>
       <c r="C79" s="8">
         <v>1</v>
       </c>
@@ -1772,7 +1788,7 @@
     </row>
     <row r="80" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="10"/>
-      <c r="B80" s="33"/>
+      <c r="B80" s="29"/>
       <c r="C80" s="10">
         <v>1</v>
       </c>
@@ -1783,7 +1799,7 @@
       <c r="A81" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B81" s="33"/>
+      <c r="B81" s="29"/>
       <c r="C81" s="22">
         <f>SUM(C76:C80)</f>
         <v>5</v>
@@ -1795,7 +1811,7 @@
       <c r="A82" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B82" s="34"/>
+      <c r="B82" s="30"/>
       <c r="C82" s="25"/>
       <c r="D82" s="26"/>
       <c r="E82" s="27"/>
@@ -1804,7 +1820,7 @@
       <c r="A83" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B83" s="32"/>
+      <c r="B83" s="28"/>
       <c r="C83" s="5">
         <v>1</v>
       </c>
@@ -1813,7 +1829,7 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="7"/>
-      <c r="B84" s="33"/>
+      <c r="B84" s="29"/>
       <c r="C84" s="8">
         <v>1</v>
       </c>
@@ -1822,7 +1838,7 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="7"/>
-      <c r="B85" s="33"/>
+      <c r="B85" s="29"/>
       <c r="C85" s="8">
         <v>1</v>
       </c>
@@ -1831,7 +1847,7 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="7"/>
-      <c r="B86" s="33"/>
+      <c r="B86" s="29"/>
       <c r="C86" s="8">
         <v>1</v>
       </c>
@@ -1840,7 +1856,7 @@
     </row>
     <row r="87" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="10"/>
-      <c r="B87" s="33"/>
+      <c r="B87" s="29"/>
       <c r="C87" s="10">
         <v>1</v>
       </c>
@@ -1851,7 +1867,7 @@
       <c r="A88" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B88" s="33"/>
+      <c r="B88" s="29"/>
       <c r="C88" s="22">
         <f>SUM(C83:C87)</f>
         <v>5</v>
@@ -1863,19 +1879,19 @@
       <c r="A89" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B89" s="34"/>
+      <c r="B89" s="30"/>
       <c r="C89" s="25"/>
       <c r="D89" s="26"/>
       <c r="E89" s="27"/>
     </row>
     <row r="90" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="35" t="s">
+      <c r="A90" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="B90" s="36"/>
+      <c r="B90" s="32"/>
       <c r="C90" s="13">
         <f>MROUND(SUM(C6:C89) /8,0.2)</f>
-        <v>25.6</v>
+        <v>27</v>
       </c>
       <c r="D90" s="14"/>
       <c r="E90" s="15"/>
@@ -1890,31 +1906,6 @@
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="D81:E81"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="B83:B89"/>
-    <mergeCell ref="D88:E88"/>
-    <mergeCell ref="C89:E89"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="B69:B75"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="C75:E75"/>
-    <mergeCell ref="B27:B33"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="A90:B90"/>
-    <mergeCell ref="B34:B40"/>
-    <mergeCell ref="B41:B47"/>
-    <mergeCell ref="B48:B54"/>
-    <mergeCell ref="B55:B61"/>
-    <mergeCell ref="B62:B68"/>
-    <mergeCell ref="B76:B82"/>
     <mergeCell ref="D60:E60"/>
     <mergeCell ref="C61:E61"/>
     <mergeCell ref="B1:C1"/>
@@ -1931,6 +1922,31 @@
     <mergeCell ref="B20:B26"/>
     <mergeCell ref="D25:E25"/>
     <mergeCell ref="C26:E26"/>
+    <mergeCell ref="A90:B90"/>
+    <mergeCell ref="B34:B40"/>
+    <mergeCell ref="B41:B47"/>
+    <mergeCell ref="B48:B54"/>
+    <mergeCell ref="B55:B61"/>
+    <mergeCell ref="B62:B68"/>
+    <mergeCell ref="B76:B82"/>
+    <mergeCell ref="B27:B33"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="C47:E47"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="B69:B75"/>
+    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="C75:E75"/>
+    <mergeCell ref="D81:E81"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="B83:B89"/>
+    <mergeCell ref="D88:E88"/>
+    <mergeCell ref="C89:E89"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C11 B13 C13:C18 B20 C20:C25 B27 C27:C32 B34 C34:C39 B41 C41:C46 B48 C48:C53 B55 C55:C60 B62 C62:C67 B69 C69:C74 B76 C76:C81 B83 C83:C88" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -1949,18 +1965,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2126,18 +2142,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
feat(compte VIP, heritage): j'ai fini l'heritage
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-RayanSahbani-jnltrav.xlsx
+++ b/doc/P-P_OO-RayanSahbani-jnltrav.xlsx
@@ -5,10 +5,10 @@
   <workbookPr updateLinks="never" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETML FID1\I320\Projet\OO-them-ALL\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETMLFID1\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4179F20D-2A2D-468F-9909-58337BDE5DA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4B0C5EA-2450-487B-A103-51A222C948D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="61">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -218,6 +218,21 @@
   </si>
   <si>
     <t>J'ai fais l'encapsulation.</t>
+  </si>
+  <si>
+    <t>J'ai commencé à faire l'heritage (TransactionVIP)</t>
+  </si>
+  <si>
+    <t>J'ai eu plusieurs problèmes dans mon code à cause de l'héritage (menu appellait plusieurs fois ainsi que des problème avec public et private)</t>
+  </si>
+  <si>
+    <t>J'ai fini l'heritage</t>
+  </si>
+  <si>
+    <t>Absence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'étais absent </t>
   </si>
 </sst>
 </file>
@@ -562,6 +577,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -579,18 +606,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -925,10 +940,10 @@
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="33"/>
+      <c r="C1" s="28"/>
       <c r="D1" s="20" t="s">
         <v>1</v>
       </c>
@@ -940,10 +955,10 @@
       <c r="A2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="33"/>
+      <c r="C2" s="28"/>
       <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
@@ -955,10 +970,10 @@
       <c r="A3" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="33"/>
+      <c r="C3" s="28"/>
       <c r="D3" s="20" t="s">
         <v>6</v>
       </c>
@@ -970,12 +985,12 @@
       <c r="A4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="36"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="31"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -998,7 +1013,7 @@
       <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="28">
+      <c r="B6" s="32">
         <v>46036</v>
       </c>
       <c r="C6" s="5">
@@ -1013,7 +1028,7 @@
       <c r="A7" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="29"/>
+      <c r="B7" s="33"/>
       <c r="C7" s="8">
         <v>3</v>
       </c>
@@ -1026,7 +1041,7 @@
       <c r="A8" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="29"/>
+      <c r="B8" s="33"/>
       <c r="C8" s="8">
         <v>1</v>
       </c>
@@ -1039,7 +1054,7 @@
       <c r="A9" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="29"/>
+      <c r="B9" s="33"/>
       <c r="C9" s="8">
         <v>2</v>
       </c>
@@ -1052,7 +1067,7 @@
       <c r="A10" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="29"/>
+      <c r="B10" s="33"/>
       <c r="C10" s="10">
         <v>3</v>
       </c>
@@ -1065,7 +1080,7 @@
       <c r="A11" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="29"/>
+      <c r="B11" s="33"/>
       <c r="C11" s="22">
         <f>SUM(C6:C10)</f>
         <v>12</v>
@@ -1077,7 +1092,7 @@
       <c r="A12" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="30"/>
+      <c r="B12" s="34"/>
       <c r="C12" s="25"/>
       <c r="D12" s="26"/>
       <c r="E12" s="27"/>
@@ -1086,7 +1101,7 @@
       <c r="A13" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="28">
+      <c r="B13" s="32">
         <v>46043</v>
       </c>
       <c r="C13" s="5">
@@ -1101,7 +1116,7 @@
       <c r="A14" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="29"/>
+      <c r="B14" s="33"/>
       <c r="C14" s="8">
         <v>5</v>
       </c>
@@ -1114,7 +1129,7 @@
       <c r="A15" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="29"/>
+      <c r="B15" s="33"/>
       <c r="C15" s="8">
         <v>4</v>
       </c>
@@ -1127,7 +1142,7 @@
       <c r="A16" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="29"/>
+      <c r="B16" s="33"/>
       <c r="C16" s="8">
         <v>1</v>
       </c>
@@ -1138,7 +1153,7 @@
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="10"/>
-      <c r="B17" s="29"/>
+      <c r="B17" s="33"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1147,7 +1162,7 @@
       <c r="A18" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="29"/>
+      <c r="B18" s="33"/>
       <c r="C18" s="22">
         <f>SUM(C13:C17)</f>
         <v>12</v>
@@ -1159,7 +1174,7 @@
       <c r="A19" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="30"/>
+      <c r="B19" s="34"/>
       <c r="C19" s="25"/>
       <c r="D19" s="26"/>
       <c r="E19" s="27"/>
@@ -1168,7 +1183,7 @@
       <c r="A20" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B20" s="28">
+      <c r="B20" s="32">
         <v>46050</v>
       </c>
       <c r="C20" s="5">
@@ -1183,7 +1198,7 @@
       <c r="A21" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="29"/>
+      <c r="B21" s="33"/>
       <c r="C21" s="8">
         <v>3</v>
       </c>
@@ -1194,7 +1209,7 @@
     </row>
     <row r="22" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
-      <c r="B22" s="29"/>
+      <c r="B22" s="33"/>
       <c r="C22" s="8">
         <v>2</v>
       </c>
@@ -1205,7 +1220,7 @@
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
-      <c r="B23" s="29"/>
+      <c r="B23" s="33"/>
       <c r="C23" s="8">
         <v>2</v>
       </c>
@@ -1216,7 +1231,7 @@
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="10"/>
-      <c r="B24" s="29"/>
+      <c r="B24" s="33"/>
       <c r="C24" s="10"/>
       <c r="D24" s="11"/>
       <c r="E24" s="10"/>
@@ -1225,7 +1240,7 @@
       <c r="A25" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="29"/>
+      <c r="B25" s="33"/>
       <c r="C25" s="22">
         <f>SUM(C20:C24)</f>
         <v>12</v>
@@ -1237,7 +1252,7 @@
       <c r="A26" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="30"/>
+      <c r="B26" s="34"/>
       <c r="C26" s="25"/>
       <c r="D26" s="26"/>
       <c r="E26" s="27"/>
@@ -1246,7 +1261,7 @@
       <c r="A27" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="28">
+      <c r="B27" s="32">
         <v>46057</v>
       </c>
       <c r="C27" s="5">
@@ -1261,7 +1276,7 @@
       <c r="A28" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B28" s="29"/>
+      <c r="B28" s="33"/>
       <c r="C28" s="8">
         <v>3</v>
       </c>
@@ -1274,7 +1289,7 @@
       <c r="A29" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B29" s="29"/>
+      <c r="B29" s="33"/>
       <c r="C29" s="8">
         <v>4</v>
       </c>
@@ -1285,14 +1300,14 @@
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
-      <c r="B30" s="29"/>
+      <c r="B30" s="33"/>
       <c r="C30" s="8"/>
       <c r="D30" s="9"/>
       <c r="E30" s="8"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="10"/>
-      <c r="B31" s="29"/>
+      <c r="B31" s="33"/>
       <c r="C31" s="10">
         <v>3</v>
       </c>
@@ -1305,7 +1320,7 @@
       <c r="A32" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B32" s="29"/>
+      <c r="B32" s="33"/>
       <c r="C32" s="22">
         <f>SUM(C27:C31)</f>
         <v>12</v>
@@ -1317,7 +1332,7 @@
       <c r="A33" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B33" s="30"/>
+      <c r="B33" s="34"/>
       <c r="C33" s="25"/>
       <c r="D33" s="26"/>
       <c r="E33" s="27"/>
@@ -1326,7 +1341,7 @@
       <c r="A34" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B34" s="28">
+      <c r="B34" s="32">
         <v>46062</v>
       </c>
       <c r="C34" s="5">
@@ -1341,7 +1356,7 @@
       <c r="A35" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B35" s="29"/>
+      <c r="B35" s="33"/>
       <c r="C35" s="8">
         <v>5</v>
       </c>
@@ -1354,7 +1369,7 @@
       <c r="A36" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B36" s="29"/>
+      <c r="B36" s="33"/>
       <c r="C36" s="8">
         <v>4</v>
       </c>
@@ -1365,14 +1380,14 @@
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
-      <c r="B37" s="29"/>
+      <c r="B37" s="33"/>
       <c r="C37" s="8"/>
       <c r="D37" s="9"/>
       <c r="E37" s="8"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="10"/>
-      <c r="B38" s="29"/>
+      <c r="B38" s="33"/>
       <c r="C38" s="10"/>
       <c r="D38" s="11"/>
       <c r="E38" s="10"/>
@@ -1381,7 +1396,7 @@
       <c r="A39" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B39" s="29"/>
+      <c r="B39" s="33"/>
       <c r="C39" s="22">
         <f>SUM(C34:C38)</f>
         <v>12</v>
@@ -1393,7 +1408,7 @@
       <c r="A40" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="30"/>
+      <c r="B40" s="34"/>
       <c r="C40" s="25"/>
       <c r="D40" s="26"/>
       <c r="E40" s="27"/>
@@ -1402,7 +1417,7 @@
       <c r="A41" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B41" s="28">
+      <c r="B41" s="32">
         <v>46064</v>
       </c>
       <c r="C41" s="5">
@@ -1417,7 +1432,7 @@
       <c r="A42" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B42" s="29"/>
+      <c r="B42" s="33"/>
       <c r="C42" s="8">
         <v>4</v>
       </c>
@@ -1428,7 +1443,7 @@
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7"/>
-      <c r="B43" s="29"/>
+      <c r="B43" s="33"/>
       <c r="C43" s="8">
         <v>5</v>
       </c>
@@ -1439,14 +1454,14 @@
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="7"/>
-      <c r="B44" s="29"/>
+      <c r="B44" s="33"/>
       <c r="C44" s="8"/>
       <c r="D44" s="9"/>
       <c r="E44" s="8"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="10"/>
-      <c r="B45" s="29"/>
+      <c r="B45" s="33"/>
       <c r="C45" s="10"/>
       <c r="D45" s="11"/>
       <c r="E45" s="10"/>
@@ -1455,7 +1470,7 @@
       <c r="A46" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B46" s="29"/>
+      <c r="B46" s="33"/>
       <c r="C46" s="22">
         <f>SUM(C41:C45)</f>
         <v>12</v>
@@ -1467,7 +1482,7 @@
       <c r="A47" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B47" s="30"/>
+      <c r="B47" s="34"/>
       <c r="C47" s="25"/>
       <c r="D47" s="26"/>
       <c r="E47" s="27"/>
@@ -1476,7 +1491,7 @@
       <c r="A48" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B48" s="28">
+      <c r="B48" s="32">
         <v>46076</v>
       </c>
       <c r="C48" s="5">
@@ -1489,28 +1504,28 @@
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
-      <c r="B49" s="29"/>
+      <c r="B49" s="33"/>
       <c r="C49" s="8"/>
       <c r="D49" s="9"/>
       <c r="E49" s="8"/>
     </row>
     <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
-      <c r="B50" s="29"/>
+      <c r="B50" s="33"/>
       <c r="C50" s="8"/>
       <c r="D50" s="9"/>
       <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="7"/>
-      <c r="B51" s="29"/>
+      <c r="B51" s="33"/>
       <c r="C51" s="8"/>
       <c r="D51" s="9"/>
       <c r="E51" s="8"/>
     </row>
     <row r="52" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="10"/>
-      <c r="B52" s="29"/>
+      <c r="B52" s="33"/>
       <c r="C52" s="10"/>
       <c r="D52" s="11"/>
       <c r="E52" s="10"/>
@@ -1519,7 +1534,7 @@
       <c r="A53" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B53" s="29"/>
+      <c r="B53" s="33"/>
       <c r="C53" s="22">
         <f>SUM(C48:C52)</f>
         <v>4</v>
@@ -1531,7 +1546,7 @@
       <c r="A54" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B54" s="30"/>
+      <c r="B54" s="34"/>
       <c r="C54" s="25"/>
       <c r="D54" s="26"/>
       <c r="E54" s="27"/>
@@ -1540,7 +1555,7 @@
       <c r="A55" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B55" s="28">
+      <c r="B55" s="32">
         <v>46078</v>
       </c>
       <c r="C55" s="5">
@@ -1555,7 +1570,7 @@
       <c r="A56" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B56" s="29"/>
+      <c r="B56" s="33"/>
       <c r="C56" s="8">
         <v>4</v>
       </c>
@@ -1568,7 +1583,7 @@
       <c r="A57" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B57" s="29"/>
+      <c r="B57" s="33"/>
       <c r="C57" s="8">
         <v>4</v>
       </c>
@@ -1579,14 +1594,14 @@
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="29"/>
+      <c r="B58" s="33"/>
       <c r="C58" s="8"/>
       <c r="D58" s="9"/>
       <c r="E58" s="8"/>
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="10"/>
-      <c r="B59" s="29"/>
+      <c r="B59" s="33"/>
       <c r="C59" s="10"/>
       <c r="D59" s="11"/>
       <c r="E59" s="10"/>
@@ -1595,7 +1610,7 @@
       <c r="A60" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B60" s="29"/>
+      <c r="B60" s="33"/>
       <c r="C60" s="22">
         <f>SUM(C55:C59)</f>
         <v>12</v>
@@ -1607,55 +1622,51 @@
       <c r="A61" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B61" s="30"/>
+      <c r="B61" s="34"/>
       <c r="C61" s="25"/>
       <c r="D61" s="26"/>
       <c r="E61" s="27"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B62" s="32">
+        <v>46085</v>
+      </c>
+      <c r="C62" s="5">
         <v>12</v>
       </c>
-      <c r="B62" s="28"/>
-      <c r="C62" s="5">
-        <v>1</v>
-      </c>
-      <c r="D62" s="6"/>
+      <c r="D62" s="6" t="s">
+        <v>60</v>
+      </c>
       <c r="E62" s="21"/>
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
-      <c r="B63" s="29"/>
-      <c r="C63" s="8">
-        <v>1</v>
-      </c>
+      <c r="B63" s="33"/>
+      <c r="C63" s="8"/>
       <c r="D63" s="9"/>
       <c r="E63" s="8"/>
     </row>
     <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="29"/>
-      <c r="C64" s="8">
-        <v>1</v>
-      </c>
+      <c r="B64" s="33"/>
+      <c r="C64" s="8"/>
       <c r="D64" s="9"/>
       <c r="E64" s="8"/>
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="7"/>
-      <c r="B65" s="29"/>
-      <c r="C65" s="8">
-        <v>1</v>
-      </c>
+      <c r="B65" s="33"/>
+      <c r="C65" s="8"/>
       <c r="D65" s="9"/>
       <c r="E65" s="8"/>
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="29"/>
-      <c r="C66" s="10">
-        <v>1</v>
-      </c>
+      <c r="B66" s="33"/>
+      <c r="C66" s="10"/>
       <c r="D66" s="11"/>
       <c r="E66" s="10"/>
     </row>
@@ -1663,10 +1674,10 @@
       <c r="A67" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B67" s="29"/>
+      <c r="B67" s="33"/>
       <c r="C67" s="22">
         <f>SUM(C62:C66)</f>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D67" s="23"/>
       <c r="E67" s="24"/>
@@ -1675,55 +1686,63 @@
       <c r="A68" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B68" s="30"/>
+      <c r="B68" s="34"/>
       <c r="C68" s="25"/>
       <c r="D68" s="26"/>
       <c r="E68" s="27"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B69" s="28"/>
+        <v>30</v>
+      </c>
+      <c r="B69" s="32">
+        <v>46092</v>
+      </c>
       <c r="C69" s="5">
-        <v>1</v>
-      </c>
-      <c r="D69" s="6"/>
+        <v>4</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>56</v>
+      </c>
       <c r="E69" s="21"/>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="7"/>
-      <c r="B70" s="29"/>
+    <row r="70" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A70" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B70" s="33"/>
       <c r="C70" s="8">
-        <v>1</v>
-      </c>
-      <c r="D70" s="9"/>
+        <v>6</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>57</v>
+      </c>
       <c r="E70" s="8"/>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="7"/>
-      <c r="B71" s="29"/>
+      <c r="A71" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B71" s="33"/>
       <c r="C71" s="8">
-        <v>1</v>
-      </c>
-      <c r="D71" s="9"/>
+        <v>2</v>
+      </c>
+      <c r="D71" s="9" t="s">
+        <v>58</v>
+      </c>
       <c r="E71" s="8"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="7"/>
-      <c r="B72" s="29"/>
-      <c r="C72" s="8">
-        <v>1</v>
-      </c>
+      <c r="B72" s="33"/>
+      <c r="C72" s="8"/>
       <c r="D72" s="9"/>
       <c r="E72" s="8"/>
     </row>
     <row r="73" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="10"/>
-      <c r="B73" s="29"/>
-      <c r="C73" s="10">
-        <v>1</v>
-      </c>
+      <c r="B73" s="33"/>
+      <c r="C73" s="10"/>
       <c r="D73" s="11"/>
       <c r="E73" s="10"/>
     </row>
@@ -1731,10 +1750,10 @@
       <c r="A74" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B74" s="29"/>
+      <c r="B74" s="33"/>
       <c r="C74" s="22">
         <f>SUM(C69:C73)</f>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D74" s="23"/>
       <c r="E74" s="24"/>
@@ -1743,7 +1762,7 @@
       <c r="A75" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B75" s="30"/>
+      <c r="B75" s="34"/>
       <c r="C75" s="25"/>
       <c r="D75" s="26"/>
       <c r="E75" s="27"/>
@@ -1752,7 +1771,7 @@
       <c r="A76" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B76" s="28"/>
+      <c r="B76" s="32"/>
       <c r="C76" s="5">
         <v>1</v>
       </c>
@@ -1761,7 +1780,7 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="7"/>
-      <c r="B77" s="29"/>
+      <c r="B77" s="33"/>
       <c r="C77" s="8">
         <v>1</v>
       </c>
@@ -1770,7 +1789,7 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="7"/>
-      <c r="B78" s="29"/>
+      <c r="B78" s="33"/>
       <c r="C78" s="8">
         <v>1</v>
       </c>
@@ -1779,7 +1798,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="7"/>
-      <c r="B79" s="29"/>
+      <c r="B79" s="33"/>
       <c r="C79" s="8">
         <v>1</v>
       </c>
@@ -1788,7 +1807,7 @@
     </row>
     <row r="80" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="10"/>
-      <c r="B80" s="29"/>
+      <c r="B80" s="33"/>
       <c r="C80" s="10">
         <v>1</v>
       </c>
@@ -1799,7 +1818,7 @@
       <c r="A81" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B81" s="29"/>
+      <c r="B81" s="33"/>
       <c r="C81" s="22">
         <f>SUM(C76:C80)</f>
         <v>5</v>
@@ -1811,7 +1830,7 @@
       <c r="A82" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B82" s="30"/>
+      <c r="B82" s="34"/>
       <c r="C82" s="25"/>
       <c r="D82" s="26"/>
       <c r="E82" s="27"/>
@@ -1820,7 +1839,7 @@
       <c r="A83" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B83" s="28"/>
+      <c r="B83" s="32"/>
       <c r="C83" s="5">
         <v>1</v>
       </c>
@@ -1829,7 +1848,7 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="7"/>
-      <c r="B84" s="29"/>
+      <c r="B84" s="33"/>
       <c r="C84" s="8">
         <v>1</v>
       </c>
@@ -1838,7 +1857,7 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="7"/>
-      <c r="B85" s="29"/>
+      <c r="B85" s="33"/>
       <c r="C85" s="8">
         <v>1</v>
       </c>
@@ -1847,7 +1866,7 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="7"/>
-      <c r="B86" s="29"/>
+      <c r="B86" s="33"/>
       <c r="C86" s="8">
         <v>1</v>
       </c>
@@ -1856,7 +1875,7 @@
     </row>
     <row r="87" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="10"/>
-      <c r="B87" s="29"/>
+      <c r="B87" s="33"/>
       <c r="C87" s="10">
         <v>1</v>
       </c>
@@ -1867,7 +1886,7 @@
       <c r="A88" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B88" s="29"/>
+      <c r="B88" s="33"/>
       <c r="C88" s="22">
         <f>SUM(C83:C87)</f>
         <v>5</v>
@@ -1879,19 +1898,19 @@
       <c r="A89" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B89" s="30"/>
+      <c r="B89" s="34"/>
       <c r="C89" s="25"/>
       <c r="D89" s="26"/>
       <c r="E89" s="27"/>
     </row>
     <row r="90" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="31" t="s">
+      <c r="A90" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="B90" s="32"/>
+      <c r="B90" s="36"/>
       <c r="C90" s="13">
         <f>MROUND(SUM(C6:C89) /8,0.2)</f>
-        <v>27</v>
+        <v>30.6</v>
       </c>
       <c r="D90" s="14"/>
       <c r="E90" s="15"/>
@@ -1906,6 +1925,31 @@
     </row>
   </sheetData>
   <mergeCells count="41">
+    <mergeCell ref="D81:E81"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="B83:B89"/>
+    <mergeCell ref="D88:E88"/>
+    <mergeCell ref="C89:E89"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="B69:B75"/>
+    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="C75:E75"/>
+    <mergeCell ref="B27:B33"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="C47:E47"/>
+    <mergeCell ref="A90:B90"/>
+    <mergeCell ref="B34:B40"/>
+    <mergeCell ref="B41:B47"/>
+    <mergeCell ref="B48:B54"/>
+    <mergeCell ref="B55:B61"/>
+    <mergeCell ref="B62:B68"/>
+    <mergeCell ref="B76:B82"/>
     <mergeCell ref="D60:E60"/>
     <mergeCell ref="C61:E61"/>
     <mergeCell ref="B1:C1"/>
@@ -1922,31 +1966,6 @@
     <mergeCell ref="B20:B26"/>
     <mergeCell ref="D25:E25"/>
     <mergeCell ref="C26:E26"/>
-    <mergeCell ref="A90:B90"/>
-    <mergeCell ref="B34:B40"/>
-    <mergeCell ref="B41:B47"/>
-    <mergeCell ref="B48:B54"/>
-    <mergeCell ref="B55:B61"/>
-    <mergeCell ref="B62:B68"/>
-    <mergeCell ref="B76:B82"/>
-    <mergeCell ref="B27:B33"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="B69:B75"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="C75:E75"/>
-    <mergeCell ref="D81:E81"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="B83:B89"/>
-    <mergeCell ref="D88:E88"/>
-    <mergeCell ref="C89:E89"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C11 B13 C13:C18 B20 C20:C25 B27 C27:C32 B34 C34:C39 B41 C41:C46 B48 C48:C53 B55 C55:C60 B62 C62:C67 B69 C69:C74 B76 C76:C81 B83 C83:C88" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -1955,7 +1974,7 @@
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="46" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="45" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -1965,18 +1984,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2142,18 +2161,18 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
feat(finalisation du rapport): fin du rapport fin du projet
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-RayanSahbani-jnltrav.xlsx
+++ b/doc/P-P_OO-RayanSahbani-jnltrav.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ETMLFID1\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4B0C5EA-2450-487B-A103-51A222C948D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C13C1C4-89A5-42AF-96EC-A23F809D19ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="63">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -233,6 +233,12 @@
   </si>
   <si>
     <t xml:space="preserve">J'étais absent </t>
+  </si>
+  <si>
+    <t>Rapport</t>
+  </si>
+  <si>
+    <t>J'ai finalisé le rapport</t>
   </si>
 </sst>
 </file>
@@ -1769,48 +1775,43 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B76" s="32"/>
+        <v>61</v>
+      </c>
+      <c r="B76" s="32">
+        <v>46094</v>
+      </c>
       <c r="C76" s="5">
-        <v>1</v>
-      </c>
-      <c r="D76" s="6"/>
+        <v>6</v>
+      </c>
+      <c r="D76" s="9" t="s">
+        <v>62</v>
+      </c>
       <c r="E76" s="21"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="7"/>
       <c r="B77" s="33"/>
-      <c r="C77" s="8">
-        <v>1</v>
-      </c>
-      <c r="D77" s="9"/>
+      <c r="C77" s="8"/>
       <c r="E77" s="8"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="7"/>
       <c r="B78" s="33"/>
-      <c r="C78" s="8">
-        <v>1</v>
-      </c>
+      <c r="C78" s="8"/>
       <c r="D78" s="9"/>
       <c r="E78" s="8"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="7"/>
       <c r="B79" s="33"/>
-      <c r="C79" s="8">
-        <v>1</v>
-      </c>
+      <c r="C79" s="8"/>
       <c r="D79" s="9"/>
       <c r="E79" s="8"/>
     </row>
     <row r="80" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="10"/>
       <c r="B80" s="33"/>
-      <c r="C80" s="10">
-        <v>1</v>
-      </c>
+      <c r="C80" s="10"/>
       <c r="D80" s="11"/>
       <c r="E80" s="10"/>
     </row>
@@ -1821,7 +1822,7 @@
       <c r="B81" s="33"/>
       <c r="C81" s="22">
         <f>SUM(C76:C80)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D81" s="23"/>
       <c r="E81" s="24"/>
@@ -1840,45 +1841,35 @@
         <v>12</v>
       </c>
       <c r="B83" s="32"/>
-      <c r="C83" s="5">
-        <v>1</v>
-      </c>
+      <c r="C83" s="5"/>
       <c r="D83" s="6"/>
       <c r="E83" s="21"/>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="7"/>
       <c r="B84" s="33"/>
-      <c r="C84" s="8">
-        <v>1</v>
-      </c>
+      <c r="C84" s="8"/>
       <c r="D84" s="9"/>
       <c r="E84" s="8"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="7"/>
       <c r="B85" s="33"/>
-      <c r="C85" s="8">
-        <v>1</v>
-      </c>
+      <c r="C85" s="8"/>
       <c r="D85" s="9"/>
       <c r="E85" s="8"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="7"/>
       <c r="B86" s="33"/>
-      <c r="C86" s="8">
-        <v>1</v>
-      </c>
+      <c r="C86" s="8"/>
       <c r="D86" s="9"/>
       <c r="E86" s="8"/>
     </row>
     <row r="87" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="10"/>
       <c r="B87" s="33"/>
-      <c r="C87" s="10">
-        <v>1</v>
-      </c>
+      <c r="C87" s="10"/>
       <c r="D87" s="11"/>
       <c r="E87" s="10"/>
     </row>
@@ -1889,7 +1880,7 @@
       <c r="B88" s="33"/>
       <c r="C88" s="22">
         <f>SUM(C83:C87)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D88" s="23"/>
       <c r="E88" s="24"/>
@@ -1910,7 +1901,7 @@
       <c r="B90" s="36"/>
       <c r="C90" s="13">
         <f>MROUND(SUM(C6:C89) /8,0.2)</f>
-        <v>30.6</v>
+        <v>29.6</v>
       </c>
       <c r="D90" s="14"/>
       <c r="E90" s="15"/>

</xml_diff>